<commit_message>
ADDED SALES ORDER HEADER QUERY IN THE TEST DATA EXCEL
ADDED SALES ORDER HEADER QUERY IN THE TEST DATA EXCEL
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="151">
   <si>
     <t>GST Sales</t>
   </si>
@@ -507,6 +507,9 @@
   </si>
   <si>
     <t>65863</t>
+  </si>
+  <si>
+    <t>65848</t>
   </si>
 </sst>
 </file>
@@ -1181,43 +1184,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -1569,8 +1572,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" s="36" t="s">
-        <v>95</v>
+      <c r="AG5" t="s" s="36">
+        <v>150</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -1769,43 +1772,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2343,44 +2346,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -2806,44 +2809,44 @@
   <dimension ref="A1:AM13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="18.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3434,44 +3437,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3897,44 +3900,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4360,43 +4363,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -4810,43 +4813,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -5260,43 +5263,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -5710,43 +5713,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -6160,43 +6163,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -6607,44 +6610,44 @@
   <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -7207,43 +7210,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -7666,42 +7669,42 @@
   <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.42578125" style="29" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="15.42578125"/>
+    <col min="38" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
@@ -8113,43 +8116,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8658,43 +8661,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9209,43 +9212,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9760,43 +9763,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10180,43 +10183,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10600,43 +10603,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="11.7109375" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="11.7109375"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -11020,44 +11023,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -11483,44 +11486,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -11946,43 +11949,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12552,43 +12555,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13140,43 +13143,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13728,43 +13731,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14316,43 +14319,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14904,43 +14907,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -15492,43 +15495,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">

</xml_diff>

<commit_message>
Newly Subcontract Order Functions Added
Newly Subcontract Order Functions Added and fixed existing
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="28" activeTab="34"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="28" activeTab="31"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1901" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1929" uniqueCount="279">
   <si>
     <t>GST Sales</t>
   </si>
@@ -373,9 +373,6 @@
     <t>HK-FIFO-LOT-BATCH-10001(FG)</t>
   </si>
   <si>
-    <t>49526</t>
-  </si>
-  <si>
     <t>Charges</t>
   </si>
   <si>
@@ -496,9 +493,6 @@
     <t>105596</t>
   </si>
   <si>
-    <t>49151</t>
-  </si>
-  <si>
     <t>64383</t>
   </si>
   <si>
@@ -535,90 +529,6 @@
     <t>Scenario  : Open SCO Price Level Type - Item + Process</t>
   </si>
   <si>
-    <t>63938</t>
-  </si>
-  <si>
-    <t>19275</t>
-  </si>
-  <si>
-    <t>63923</t>
-  </si>
-  <si>
-    <t>19270</t>
-  </si>
-  <si>
-    <t>9255</t>
-  </si>
-  <si>
-    <t>19808.992</t>
-  </si>
-  <si>
-    <t>109415</t>
-  </si>
-  <si>
-    <t>109755</t>
-  </si>
-  <si>
-    <t>9765</t>
-  </si>
-  <si>
-    <t>9307</t>
-  </si>
-  <si>
-    <t>9715</t>
-  </si>
-  <si>
-    <t>9415</t>
-  </si>
-  <si>
-    <t>9760</t>
-  </si>
-  <si>
-    <t>9293</t>
-  </si>
-  <si>
-    <t>9702.5</t>
-  </si>
-  <si>
-    <t>9425</t>
-  </si>
-  <si>
-    <t>109411</t>
-  </si>
-  <si>
-    <t>109750</t>
-  </si>
-  <si>
-    <t>109500</t>
-  </si>
-  <si>
-    <t>109785</t>
-  </si>
-  <si>
-    <t>63893</t>
-  </si>
-  <si>
-    <t>63878</t>
-  </si>
-  <si>
-    <t>63863</t>
-  </si>
-  <si>
-    <t>63848</t>
-  </si>
-  <si>
-    <t>488826</t>
-  </si>
-  <si>
-    <t>63838</t>
-  </si>
-  <si>
-    <t>18880</t>
-  </si>
-  <si>
-    <t>19265</t>
-  </si>
-  <si>
     <t>Scenario  : Open SCO Price Level Type - Supplier + Process</t>
   </si>
   <si>
@@ -640,27 +550,12 @@
     <t>7</t>
   </si>
   <si>
-    <t>63823</t>
-  </si>
-  <si>
-    <t>19257.5</t>
-  </si>
-  <si>
     <t>63808</t>
   </si>
   <si>
     <t>19252.5</t>
   </si>
   <si>
-    <t>9240</t>
-  </si>
-  <si>
-    <t>19803.992</t>
-  </si>
-  <si>
-    <t>109400</t>
-  </si>
-  <si>
     <t>63793</t>
   </si>
   <si>
@@ -679,39 +574,15 @@
     <t>109745</t>
   </si>
   <si>
-    <t>9292</t>
-  </si>
-  <si>
-    <t>9710</t>
-  </si>
-  <si>
-    <t>9400</t>
-  </si>
-  <si>
     <t>9755</t>
   </si>
   <si>
-    <t>9277</t>
-  </si>
-  <si>
-    <t>9705</t>
-  </si>
-  <si>
     <t>9385</t>
   </si>
   <si>
     <t>9750</t>
   </si>
   <si>
-    <t>9278</t>
-  </si>
-  <si>
-    <t>9697.5</t>
-  </si>
-  <si>
-    <t>9410</t>
-  </si>
-  <si>
     <t>9263</t>
   </si>
   <si>
@@ -721,15 +592,6 @@
     <t>9395</t>
   </si>
   <si>
-    <t>109396</t>
-  </si>
-  <si>
-    <t>109485</t>
-  </si>
-  <si>
-    <t>109780</t>
-  </si>
-  <si>
     <t>109381</t>
   </si>
   <si>
@@ -742,9 +604,6 @@
     <t>109775</t>
   </si>
   <si>
-    <t>63778</t>
-  </si>
-  <si>
     <t>63763</t>
   </si>
   <si>
@@ -775,40 +634,271 @@
     <t>9700</t>
   </si>
   <si>
-    <t>63693</t>
-  </si>
-  <si>
-    <t>63678</t>
-  </si>
-  <si>
-    <t>63663</t>
-  </si>
-  <si>
-    <t>49136</t>
-  </si>
-  <si>
     <t>49121</t>
   </si>
   <si>
-    <t>49106</t>
-  </si>
-  <si>
     <t>49091</t>
   </si>
   <si>
-    <t>63648</t>
-  </si>
-  <si>
-    <t>63633</t>
-  </si>
-  <si>
-    <t>63618</t>
-  </si>
-  <si>
-    <t>63603</t>
-  </si>
-  <si>
     <t>63588</t>
+  </si>
+  <si>
+    <t>63573</t>
+  </si>
+  <si>
+    <t>19235</t>
+  </si>
+  <si>
+    <t>9210</t>
+  </si>
+  <si>
+    <t>19793.992</t>
+  </si>
+  <si>
+    <t>63558</t>
+  </si>
+  <si>
+    <t>19230</t>
+  </si>
+  <si>
+    <t>9195</t>
+  </si>
+  <si>
+    <t>19788.992</t>
+  </si>
+  <si>
+    <t>9247</t>
+  </si>
+  <si>
+    <t>9695</t>
+  </si>
+  <si>
+    <t>9232</t>
+  </si>
+  <si>
+    <t>9690</t>
+  </si>
+  <si>
+    <t>9248</t>
+  </si>
+  <si>
+    <t>9687.5</t>
+  </si>
+  <si>
+    <t>9233</t>
+  </si>
+  <si>
+    <t>9682.5</t>
+  </si>
+  <si>
+    <t>109366</t>
+  </si>
+  <si>
+    <t>109735</t>
+  </si>
+  <si>
+    <t>109351</t>
+  </si>
+  <si>
+    <t>109730</t>
+  </si>
+  <si>
+    <t>63543</t>
+  </si>
+  <si>
+    <t>63528</t>
+  </si>
+  <si>
+    <t>63513</t>
+  </si>
+  <si>
+    <t>63498</t>
+  </si>
+  <si>
+    <t>488806</t>
+  </si>
+  <si>
+    <t>63488</t>
+  </si>
+  <si>
+    <t>18850</t>
+  </si>
+  <si>
+    <t>19225</t>
+  </si>
+  <si>
+    <t>63473</t>
+  </si>
+  <si>
+    <t>63458</t>
+  </si>
+  <si>
+    <t>63443</t>
+  </si>
+  <si>
+    <t>49076</t>
+  </si>
+  <si>
+    <t>63428</t>
+  </si>
+  <si>
+    <t>63413</t>
+  </si>
+  <si>
+    <t>63398</t>
+  </si>
+  <si>
+    <t>63383</t>
+  </si>
+  <si>
+    <t>63368</t>
+  </si>
+  <si>
+    <t>63338</t>
+  </si>
+  <si>
+    <t>63323</t>
+  </si>
+  <si>
+    <t>63308</t>
+  </si>
+  <si>
+    <t>63293</t>
+  </si>
+  <si>
+    <t>63278</t>
+  </si>
+  <si>
+    <t>63263</t>
+  </si>
+  <si>
+    <t>49061</t>
+  </si>
+  <si>
+    <t>63248</t>
+  </si>
+  <si>
+    <t>63233</t>
+  </si>
+  <si>
+    <t>63218</t>
+  </si>
+  <si>
+    <t>63203</t>
+  </si>
+  <si>
+    <t>63188</t>
+  </si>
+  <si>
+    <t>63173</t>
+  </si>
+  <si>
+    <t>63158</t>
+  </si>
+  <si>
+    <t>63143</t>
+  </si>
+  <si>
+    <t>63128</t>
+  </si>
+  <si>
+    <t>63113</t>
+  </si>
+  <si>
+    <t>63098</t>
+  </si>
+  <si>
+    <t>63083</t>
+  </si>
+  <si>
+    <t>63068</t>
+  </si>
+  <si>
+    <t>63053</t>
+  </si>
+  <si>
+    <t>63038</t>
+  </si>
+  <si>
+    <t>63023</t>
+  </si>
+  <si>
+    <t>63008</t>
+  </si>
+  <si>
+    <t>62993</t>
+  </si>
+  <si>
+    <t>62978</t>
+  </si>
+  <si>
+    <t>19217.5</t>
+  </si>
+  <si>
+    <t>9180</t>
+  </si>
+  <si>
+    <t>19783.992</t>
+  </si>
+  <si>
+    <t>62963</t>
+  </si>
+  <si>
+    <t>19212.5</t>
+  </si>
+  <si>
+    <t>9165</t>
+  </si>
+  <si>
+    <t>19778.992</t>
+  </si>
+  <si>
+    <t>9217</t>
+  </si>
+  <si>
+    <t>9685</t>
+  </si>
+  <si>
+    <t>9202</t>
+  </si>
+  <si>
+    <t>9680</t>
+  </si>
+  <si>
+    <t>9218</t>
+  </si>
+  <si>
+    <t>9677.5</t>
+  </si>
+  <si>
+    <t>9203</t>
+  </si>
+  <si>
+    <t>9672.5</t>
+  </si>
+  <si>
+    <t>109336</t>
+  </si>
+  <si>
+    <t>109725</t>
+  </si>
+  <si>
+    <t>109321</t>
+  </si>
+  <si>
+    <t>109720</t>
+  </si>
+  <si>
+    <t>62948</t>
+  </si>
+  <si>
+    <t>49046</t>
+  </si>
+  <si>
+    <t>49031</t>
+  </si>
+  <si>
+    <t>62933</t>
   </si>
 </sst>
 </file>
@@ -1952,7 +2042,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>199</v>
+        <v>259</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -2081,7 +2171,7 @@
         <v>5</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>200</v>
+        <v>260</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -2449,7 +2539,7 @@
       <c r="G5" s="33">
         <v>15</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>77</v>
       </c>
       <c r="I5" s="9">
@@ -2535,8 +2625,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>224</v>
+      <c r="AG5" s="36" t="s">
+        <v>178</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -2573,7 +2663,7 @@
       <c r="G6" s="33">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="29">
+      <c r="H6" s="29" t="s">
         <v>78</v>
       </c>
       <c r="I6" s="9">
@@ -2659,8 +2749,8 @@
         <f>ROUND(G6/AE6,3)</f>
         <v>5</v>
       </c>
-      <c r="AG6" t="s" s="36">
-        <v>225</v>
+      <c r="AG6" s="36" t="s">
+        <v>179</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -3116,7 +3206,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -3578,8 +3668,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" s="36" t="s">
-        <v>145</v>
+      <c r="AG5" t="s" s="36">
+        <v>246</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -3638,7 +3728,7 @@
     </row>
     <row r="9" spans="1:39">
       <c r="C9" s="89" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9" s="23"/>
       <c r="E9" s="23"/>
@@ -3655,7 +3745,7 @@
     </row>
     <row r="10" spans="1:39">
       <c r="C10" s="90" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D10" s="90" t="s">
         <v>6</v>
@@ -3664,19 +3754,19 @@
         <v>7</v>
       </c>
       <c r="F10" s="90" t="s">
+        <v>105</v>
+      </c>
+      <c r="G10" s="90" t="s">
         <v>106</v>
       </c>
-      <c r="G10" s="90" t="s">
+      <c r="H10" s="90" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="90" t="s">
+      <c r="I10" s="90" t="s">
         <v>108</v>
       </c>
-      <c r="I10" s="90" t="s">
+      <c r="J10" s="90" t="s">
         <v>109</v>
-      </c>
-      <c r="J10" s="90" t="s">
-        <v>110</v>
       </c>
       <c r="K10" s="90" t="s">
         <v>26</v>
@@ -3699,16 +3789,16 @@
         <v>1</v>
       </c>
       <c r="D11" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E11" s="10">
+        <v>0</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="E11" s="10">
-        <v>0</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>113</v>
       </c>
       <c r="H11" s="10">
         <v>20</v>
@@ -3740,16 +3830,16 @@
         <v>2</v>
       </c>
       <c r="D12" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="E12" s="10">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>115</v>
-      </c>
       <c r="G12" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H12" s="10"/>
       <c r="I12" s="10">
@@ -3781,7 +3871,7 @@
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I13" s="10">
         <v>21477.41</v>
@@ -4103,13 +4193,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -4207,7 +4297,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -4670,7 +4760,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -4697,13 +4787,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="97" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="97" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -4801,7 +4891,7 @@
         <v>16</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AH6" s="34">
         <f>AG6-AF6</f>
@@ -4827,13 +4917,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="97" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" s="10">
         <v>0</v>
       </c>
       <c r="D7" s="97" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>32</v>
@@ -4931,7 +5021,7 @@
         <v>17</v>
       </c>
       <c r="AG7" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AH7" s="34">
         <f t="shared" ref="AH7:AH14" si="20">AG7-AF7</f>
@@ -4957,13 +5047,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="97" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
       </c>
       <c r="D8" s="97" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>32</v>
@@ -5061,7 +5151,7 @@
         <v>18</v>
       </c>
       <c r="AG8" s="36" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AH8" s="34">
         <f t="shared" si="20"/>
@@ -5087,13 +5177,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="97" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
       </c>
       <c r="D9" s="97" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>32</v>
@@ -5191,7 +5281,7 @@
         <v>19</v>
       </c>
       <c r="AG9" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AH9" s="34">
         <f t="shared" si="20"/>
@@ -5217,13 +5307,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="97" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
       </c>
       <c r="D10" s="97" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>32</v>
@@ -5321,7 +5411,7 @@
         <v>20</v>
       </c>
       <c r="AG10" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AH10" s="34">
         <f t="shared" si="20"/>
@@ -5347,13 +5437,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="97" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C11" s="10">
         <v>0</v>
       </c>
       <c r="D11" s="97" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>32</v>
@@ -5451,7 +5541,7 @@
         <v>21</v>
       </c>
       <c r="AG11" s="36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AH11" s="34">
         <f t="shared" si="20"/>
@@ -5477,13 +5567,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C12" s="99">
         <v>0</v>
       </c>
       <c r="D12" s="100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E12" s="99" t="s">
         <v>32</v>
@@ -5581,7 +5671,7 @@
         <v>22</v>
       </c>
       <c r="AG12" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AH12" s="102">
         <f t="shared" si="20"/>
@@ -5607,13 +5697,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="97" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C13" s="10">
         <v>0</v>
       </c>
       <c r="D13" s="97" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>32</v>
@@ -5711,7 +5801,7 @@
         <v>23</v>
       </c>
       <c r="AG13" s="36" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AH13" s="34">
         <f t="shared" si="20"/>
@@ -5737,13 +5827,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="97" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C14" s="10">
         <v>0</v>
       </c>
       <c r="D14" s="97" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>32</v>
@@ -5841,7 +5931,7 @@
         <v>24</v>
       </c>
       <c r="AG14" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AH14" s="34">
         <f t="shared" si="20"/>
@@ -6894,19 +6984,19 @@
         <v>100</v>
       </c>
       <c r="AM4" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="AN4" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="AO4" s="98" t="s">
         <v>129</v>
       </c>
-      <c r="AN4" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="AO4" s="98" t="s">
+      <c r="AP4" s="98" t="s">
         <v>130</v>
       </c>
-      <c r="AP4" s="98" t="s">
+      <c r="AQ4" s="98" t="s">
         <v>131</v>
-      </c>
-      <c r="AQ4" s="98" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="15">
@@ -7018,7 +7108,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>248</v>
+        <v>278</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -7042,10 +7132,10 @@
         <v>79</v>
       </c>
       <c r="AN5" s="67" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AO5" s="29" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -7491,7 +7581,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>227</v>
+        <v>214</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -7941,7 +8031,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -8391,7 +8481,7 @@
         <v>10</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -8841,7 +8931,7 @@
         <v>10</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -9299,7 +9389,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>194</v>
+        <v>275</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -9431,8 +9521,8 @@
         <f>ROUND(G6/AE6,3)</f>
         <v>5</v>
       </c>
-      <c r="AG6" t="s" s="36">
-        <v>195</v>
+      <c r="AG6" s="36" t="s">
+        <v>163</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -10794,8 +10884,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>228</v>
+      <c r="AG5" s="36" t="s">
+        <v>181</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -11246,7 +11336,7 @@
         <v>7.5</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -11372,7 +11462,7 @@
         <v>15</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -14156,8 +14246,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>243</v>
+      <c r="AG5" s="36" t="s">
+        <v>191</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -14618,7 +14708,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>201</v>
+        <v>261</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -14747,7 +14837,7 @@
         <v>5</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>202</v>
+        <v>262</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -15208,7 +15298,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>241</v>
+        <v>277</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -15290,7 +15380,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="122" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B1" s="122"/>
       <c r="C1" s="122"/>
@@ -15311,13 +15401,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>148</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15326,13 +15416,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
       </c>
       <c r="D5" s="112" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="59"/>
     </row>
@@ -15341,7 +15431,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C6" s="10">
         <v>3</v>
@@ -15375,7 +15465,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="122" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B1" s="122"/>
       <c r="C1" s="122"/>
@@ -15396,13 +15486,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>148</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15411,13 +15501,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
       </c>
       <c r="D5" s="112" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="59"/>
     </row>
@@ -15426,7 +15516,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C6" s="10">
         <v>3</v>
@@ -15460,7 +15550,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="122" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="B1" s="122"/>
       <c r="C1" s="122"/>
@@ -15481,13 +15571,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>148</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15496,13 +15586,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
       </c>
       <c r="D5" s="112" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="59"/>
     </row>
@@ -15511,7 +15601,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C6" s="10">
         <v>3</v>
@@ -15545,7 +15635,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="122" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="B1" s="122"/>
       <c r="C1" s="122"/>
@@ -15566,13 +15656,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>148</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15581,13 +15671,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
       </c>
       <c r="D5" s="112" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="59"/>
     </row>
@@ -15596,7 +15686,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C6" s="10">
         <v>3</v>
@@ -15630,7 +15720,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="122" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="B1" s="122"/>
       <c r="C1" s="122"/>
@@ -15653,10 +15743,10 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15665,13 +15755,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>191</v>
+        <v>161</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="E5" s="59"/>
     </row>
@@ -16001,7 +16091,7 @@
       <c r="G5" s="33">
         <v>15</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>62</v>
       </c>
       <c r="I5" s="9">
@@ -16087,8 +16177,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>203</v>
+      <c r="AG5" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -16130,7 +16220,7 @@
       <c r="G6" s="33">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="29">
+      <c r="H6" s="29" t="s">
         <v>54</v>
       </c>
       <c r="I6" s="9">
@@ -16216,8 +16306,8 @@
         <f>ROUND(G6/AE6,3)</f>
         <v>5</v>
       </c>
-      <c r="AG6" t="s" s="36">
-        <v>204</v>
+      <c r="AG6" s="36" t="s">
+        <v>169</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -16676,7 +16766,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>235</v>
+        <v>265</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -16805,7 +16895,7 @@
         <v>5</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -17177,7 +17267,7 @@
       <c r="G5" s="33">
         <v>15</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>61</v>
       </c>
       <c r="I5" s="9">
@@ -17263,8 +17353,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>211</v>
+      <c r="AG5" s="36" t="s">
+        <v>171</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -17306,7 +17396,7 @@
       <c r="G6" s="33">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="29">
+      <c r="H6" s="29" t="s">
         <v>62</v>
       </c>
       <c r="I6" s="9">
@@ -17392,8 +17482,8 @@
         <f>ROUND(G6/AE6,3)</f>
         <v>5</v>
       </c>
-      <c r="AG6" t="s" s="36">
-        <v>212</v>
+      <c r="AG6" s="36" t="s">
+        <v>172</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -17852,7 +17942,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>216</v>
+        <v>269</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -17981,7 +18071,7 @@
         <v>5</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>217</v>
+        <v>270</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -18353,7 +18443,7 @@
       <c r="G5" s="33">
         <v>15</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>69</v>
       </c>
       <c r="I5" s="9">
@@ -18439,8 +18529,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>218</v>
+      <c r="AG5" s="36" t="s">
+        <v>175</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -18482,7 +18572,7 @@
       <c r="G6" s="33">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="29">
+      <c r="H6" s="29" t="s">
         <v>70</v>
       </c>
       <c r="I6" s="9">
@@ -18568,8 +18658,8 @@
         <f>ROUND(G6/AE6,3)</f>
         <v>5</v>
       </c>
-      <c r="AG6" t="s" s="36">
-        <v>208</v>
+      <c r="AG6" s="36" t="s">
+        <v>170</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -19028,7 +19118,7 @@
         <v>15</v>
       </c>
       <c r="AG5" t="s" s="36">
-        <v>222</v>
+        <v>273</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -19157,7 +19247,7 @@
         <v>5</v>
       </c>
       <c r="AG6" t="s" s="36">
-        <v>223</v>
+        <v>274</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>

</xml_diff>

<commit_message>
In Test Data Sheet Added DB Query And Newly Added Subcontract Scenarios
In Test Data Sheet Added DB Query And Newly Added Subcontract Scenarios
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="32" activeTab="36"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="33" activeTab="36"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -43,8 +43,9 @@
     <sheet name="DirectSCOWithProject" sheetId="45" r:id="rId34"/>
     <sheet name="DirectSCOWithSOandConv" sheetId="44" r:id="rId35"/>
     <sheet name="DirectSCOWithConv" sheetId="42" r:id="rId36"/>
-    <sheet name="DirectSCO" sheetId="39" r:id="rId37"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId38"/>
+    <sheet name="DirectSCOSerial" sheetId="46" r:id="rId37"/>
+    <sheet name="DirectSCO" sheetId="39" r:id="rId38"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId39"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1823" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="203">
   <si>
     <t>GST Sales</t>
   </si>
@@ -664,6 +665,15 @@
   </si>
   <si>
     <t>VJ-PROJECT</t>
+  </si>
+  <si>
+    <t>PROC-004</t>
+  </si>
+  <si>
+    <t>VR-SERIAL-FIFO-BATCH-90001</t>
+  </si>
+  <si>
+    <t>Scenario  : Direct SCO Serial With BOM Standard Type</t>
   </si>
 </sst>
 </file>
@@ -832,7 +842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1100,6 +1110,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1449,36 +1465,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -1525,10 +1541,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2037,36 +2053,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -2113,10 +2129,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2612,36 +2628,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="80"/>
       <c r="AD1" s="80"/>
       <c r="AE1" s="80"/>
@@ -2688,10 +2704,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="79"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -3075,36 +3091,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="86"/>
       <c r="AD1" s="86"/>
       <c r="AE1" s="86"/>
@@ -3151,10 +3167,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="85"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -3703,36 +3719,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="88"/>
       <c r="AD1" s="88"/>
       <c r="AE1" s="88"/>
@@ -3779,10 +3795,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="87"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4166,36 +4182,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="93"/>
       <c r="AD1" s="93"/>
       <c r="AE1" s="93"/>
@@ -4242,10 +4258,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="92"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6500,36 +6516,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -6576,10 +6592,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6992,36 +7008,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -7068,10 +7084,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7442,36 +7458,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7518,10 +7534,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7892,36 +7908,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7968,10 +7984,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8342,36 +8358,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -8418,10 +8434,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8793,36 +8809,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="39"/>
       <c r="AD1" s="39"/>
       <c r="AE1" s="39"/>
@@ -8869,10 +8885,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="38"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -9392,36 +9408,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -9468,10 +9484,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -9839,36 +9855,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -9915,10 +9931,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -10297,36 +10313,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -10373,10 +10389,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:37" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -10745,36 +10761,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="65"/>
       <c r="AD1" s="65"/>
       <c r="AE1" s="65"/>
@@ -10821,10 +10837,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="64"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -11290,36 +11306,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="69"/>
       <c r="AD1" s="69"/>
       <c r="AE1" s="69"/>
@@ -11366,10 +11382,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -11841,36 +11857,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="71"/>
       <c r="AD1" s="71"/>
       <c r="AE1" s="71"/>
@@ -11917,10 +11933,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="70"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -12392,36 +12408,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="74"/>
       <c r="AD1" s="74"/>
       <c r="AE1" s="74"/>
@@ -12468,10 +12484,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="73"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12812,36 +12828,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="76"/>
       <c r="AD1" s="76"/>
       <c r="AE1" s="76"/>
@@ -12888,10 +12904,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="75"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13232,36 +13248,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="78"/>
       <c r="AD1" s="78"/>
       <c r="AE1" s="78"/>
@@ -13308,10 +13324,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="77"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13653,36 +13669,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="84"/>
       <c r="AD1" s="84"/>
       <c r="AE1" s="84"/>
@@ -13729,10 +13745,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="83"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -14115,36 +14131,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="41"/>
       <c r="AD1" s="41"/>
       <c r="AE1" s="41"/>
@@ -14191,10 +14207,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="40"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -14704,36 +14720,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="82"/>
       <c r="AD1" s="82"/>
       <c r="AE1" s="82"/>
@@ -14780,10 +14796,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -15135,19 +15151,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15205,19 +15221,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15276,19 +15292,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15357,19 +15373,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15438,19 +15454,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15518,19 +15534,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15592,21 +15608,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="A1" s="119" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
-      <c r="D2" s="109"/>
+      <c r="D2" s="117"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="108"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="116"/>
     </row>
     <row r="4" spans="1:5" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
@@ -15630,13 +15646,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>148</v>
+        <v>62</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="E5" s="67" t="s">
         <v>191</v>
@@ -15653,6 +15669,80 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="27.75" customHeight="1">
+      <c r="A1" s="119" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+    </row>
+    <row r="2" spans="1:5" ht="18">
+      <c r="D2" s="109"/>
+    </row>
+    <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="108"/>
+    </row>
+    <row r="4" spans="1:5" s="31" customFormat="1">
+      <c r="A4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="113" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15">
+      <c r="A5" s="10">
+        <v>1</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>191</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
@@ -15706,36 +15796,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="44"/>
       <c r="AD1" s="44"/>
       <c r="AE1" s="44"/>
@@ -15782,10 +15872,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="43"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -16294,36 +16384,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="46"/>
       <c r="AD1" s="46"/>
       <c r="AE1" s="46"/>
@@ -16370,10 +16460,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="45"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -16882,36 +16972,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="48"/>
       <c r="AD1" s="48"/>
       <c r="AE1" s="48"/>
@@ -16958,10 +17048,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="47"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -17470,36 +17560,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -17546,10 +17636,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -18058,36 +18148,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -18134,10 +18224,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -18646,36 +18736,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -18722,10 +18812,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
Revert "In Test Data Sheet Added DB Query And Newly Added Subcontract Scenarios"
This reverts commit 24d9d5b877db7b421e99d5971d89e3c4d95a6711.
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="33" activeTab="36"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="32" activeTab="36"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -43,9 +43,8 @@
     <sheet name="DirectSCOWithProject" sheetId="45" r:id="rId34"/>
     <sheet name="DirectSCOWithSOandConv" sheetId="44" r:id="rId35"/>
     <sheet name="DirectSCOWithConv" sheetId="42" r:id="rId36"/>
-    <sheet name="DirectSCOSerial" sheetId="46" r:id="rId37"/>
-    <sheet name="DirectSCO" sheetId="39" r:id="rId38"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId39"/>
+    <sheet name="DirectSCO" sheetId="39" r:id="rId37"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId38"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -65,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1823" uniqueCount="200">
   <si>
     <t>GST Sales</t>
   </si>
@@ -665,15 +664,6 @@
   </si>
   <si>
     <t>VJ-PROJECT</t>
-  </si>
-  <si>
-    <t>PROC-004</t>
-  </si>
-  <si>
-    <t>VR-SERIAL-FIFO-BATCH-90001</t>
-  </si>
-  <si>
-    <t>Scenario  : Direct SCO Serial With BOM Standard Type</t>
   </si>
 </sst>
 </file>
@@ -842,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1110,12 +1100,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1465,36 +1449,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -1541,10 +1525,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2053,36 +2037,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -2129,10 +2113,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2628,36 +2612,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="80"/>
       <c r="AD1" s="80"/>
       <c r="AE1" s="80"/>
@@ -2704,10 +2688,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="79"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -3091,36 +3075,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="86"/>
       <c r="AD1" s="86"/>
       <c r="AE1" s="86"/>
@@ -3167,10 +3151,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="85"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -3719,36 +3703,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="88"/>
       <c r="AD1" s="88"/>
       <c r="AE1" s="88"/>
@@ -3795,10 +3779,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="87"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4182,36 +4166,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="93"/>
       <c r="AD1" s="93"/>
       <c r="AE1" s="93"/>
@@ -4258,10 +4242,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="92"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6516,36 +6500,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -6592,10 +6576,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7008,36 +6992,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -7084,10 +7068,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7458,36 +7442,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7534,10 +7518,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7908,36 +7892,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7984,10 +7968,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8358,36 +8342,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -8434,10 +8418,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8809,36 +8793,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="39"/>
       <c r="AD1" s="39"/>
       <c r="AE1" s="39"/>
@@ -8885,10 +8869,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="38"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -9408,36 +9392,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -9484,10 +9468,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -9855,36 +9839,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -9931,10 +9915,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -10313,36 +10297,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -10389,10 +10373,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:37" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -10761,36 +10745,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="65"/>
       <c r="AD1" s="65"/>
       <c r="AE1" s="65"/>
@@ -10837,10 +10821,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="64"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -11306,36 +11290,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="69"/>
       <c r="AD1" s="69"/>
       <c r="AE1" s="69"/>
@@ -11382,10 +11366,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -11857,36 +11841,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="71"/>
       <c r="AD1" s="71"/>
       <c r="AE1" s="71"/>
@@ -11933,10 +11917,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="70"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -12408,36 +12392,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="74"/>
       <c r="AD1" s="74"/>
       <c r="AE1" s="74"/>
@@ -12484,10 +12468,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="73"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12828,36 +12812,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="76"/>
       <c r="AD1" s="76"/>
       <c r="AE1" s="76"/>
@@ -12904,10 +12888,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="75"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13248,36 +13232,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="78"/>
       <c r="AD1" s="78"/>
       <c r="AE1" s="78"/>
@@ -13324,10 +13308,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="77"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13669,36 +13653,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="84"/>
       <c r="AD1" s="84"/>
       <c r="AE1" s="84"/>
@@ -13745,10 +13729,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="83"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -14131,36 +14115,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="41"/>
       <c r="AD1" s="41"/>
       <c r="AE1" s="41"/>
@@ -14207,10 +14191,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="40"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -14720,36 +14704,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="82"/>
       <c r="AD1" s="82"/>
       <c r="AE1" s="82"/>
@@ -14796,10 +14780,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -15151,19 +15135,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15221,19 +15205,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15292,19 +15276,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15373,19 +15357,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15454,19 +15438,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15534,19 +15518,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15608,21 +15592,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
-        <v>202</v>
-      </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
+      <c r="A1" s="117" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
     </row>
     <row r="2" spans="1:5" ht="18">
-      <c r="D2" s="117"/>
+      <c r="D2" s="109"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
+      <c r="A3" s="116"/>
+      <c r="B3" s="116"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="108"/>
     </row>
     <row r="4" spans="1:5" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
@@ -15646,13 +15630,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>201</v>
+        <v>146</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>62</v>
+        <v>148</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>200</v>
+        <v>181</v>
       </c>
       <c r="E5" s="67" t="s">
         <v>191</v>
@@ -15669,80 +15653,6 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-    </row>
-    <row r="2" spans="1:5" ht="18">
-      <c r="D2" s="109"/>
-    </row>
-    <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118"/>
-      <c r="B3" s="118"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="108"/>
-    </row>
-    <row r="4" spans="1:5" s="31" customFormat="1">
-      <c r="A4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="E4" s="113" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15">
-      <c r="A5" s="10">
-        <v>1</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>148</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="E5" s="67" t="s">
-        <v>191</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:B3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
@@ -15796,36 +15706,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="44"/>
       <c r="AD1" s="44"/>
       <c r="AE1" s="44"/>
@@ -15872,10 +15782,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="43"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -16384,36 +16294,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="46"/>
       <c r="AD1" s="46"/>
       <c r="AE1" s="46"/>
@@ -16460,10 +16370,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="45"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -16972,36 +16882,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="48"/>
       <c r="AD1" s="48"/>
       <c r="AE1" s="48"/>
@@ -17048,10 +16958,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="47"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -17560,36 +17470,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -17636,10 +17546,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -18148,36 +18058,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -18224,10 +18134,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -18736,36 +18646,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="117" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -18812,10 +18722,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="118"/>
+      <c r="A3" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
In Test Data Sheet Added DB Query And Newly Subcontract Scenarios Added
In Test Data Sheet Added DB Query And Newly Subcontract Scenarios Added
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="32" activeTab="36"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="33" activeTab="36"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -43,8 +43,9 @@
     <sheet name="DirectSCOWithProject" sheetId="45" r:id="rId34"/>
     <sheet name="DirectSCOWithSOandConv" sheetId="44" r:id="rId35"/>
     <sheet name="DirectSCOWithConv" sheetId="42" r:id="rId36"/>
-    <sheet name="DirectSCO" sheetId="39" r:id="rId37"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId38"/>
+    <sheet name="DirectSCOSerial" sheetId="46" r:id="rId37"/>
+    <sheet name="DirectSCO" sheetId="39" r:id="rId38"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId39"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1823" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="203">
   <si>
     <t>GST Sales</t>
   </si>
@@ -664,6 +665,15 @@
   </si>
   <si>
     <t>VJ-PROJECT</t>
+  </si>
+  <si>
+    <t>PROC-004</t>
+  </si>
+  <si>
+    <t>VR-SERIAL-FIFO-BATCH-90001</t>
+  </si>
+  <si>
+    <t>Scenario  : Direct SCO Serial With BOM Standard Type</t>
   </si>
 </sst>
 </file>
@@ -832,7 +842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1100,6 +1110,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1449,36 +1465,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -1525,10 +1541,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2037,36 +2053,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -2113,10 +2129,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2612,36 +2628,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="80"/>
       <c r="AD1" s="80"/>
       <c r="AE1" s="80"/>
@@ -2688,10 +2704,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="79"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -3075,36 +3091,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="86"/>
       <c r="AD1" s="86"/>
       <c r="AE1" s="86"/>
@@ -3151,10 +3167,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="85"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -3703,36 +3719,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="88"/>
       <c r="AD1" s="88"/>
       <c r="AE1" s="88"/>
@@ -3779,10 +3795,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="87"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4166,36 +4182,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="93"/>
       <c r="AD1" s="93"/>
       <c r="AE1" s="93"/>
@@ -4242,10 +4258,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="92"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6500,36 +6516,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -6576,10 +6592,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6992,36 +7008,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -7068,10 +7084,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -7442,36 +7458,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7518,10 +7534,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7892,36 +7908,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -7968,10 +7984,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8342,36 +8358,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -8418,10 +8434,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8793,36 +8809,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="39"/>
       <c r="AD1" s="39"/>
       <c r="AE1" s="39"/>
@@ -8869,10 +8885,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="38"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -9392,36 +9408,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -9468,10 +9484,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -9839,36 +9855,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -9915,10 +9931,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -10297,36 +10313,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -10373,10 +10389,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:37" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -10745,36 +10761,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="65"/>
       <c r="AD1" s="65"/>
       <c r="AE1" s="65"/>
@@ -10821,10 +10837,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="64"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -11290,36 +11306,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="69"/>
       <c r="AD1" s="69"/>
       <c r="AE1" s="69"/>
@@ -11366,10 +11382,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -11841,36 +11857,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="71"/>
       <c r="AD1" s="71"/>
       <c r="AE1" s="71"/>
@@ -11917,10 +11933,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="70"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -12392,36 +12408,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="74"/>
       <c r="AD1" s="74"/>
       <c r="AE1" s="74"/>
@@ -12468,10 +12484,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="73"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12812,36 +12828,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="76"/>
       <c r="AD1" s="76"/>
       <c r="AE1" s="76"/>
@@ -12888,10 +12904,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="75"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13232,36 +13248,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="78"/>
       <c r="AD1" s="78"/>
       <c r="AE1" s="78"/>
@@ -13308,10 +13324,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="77"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -13653,36 +13669,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="84"/>
       <c r="AD1" s="84"/>
       <c r="AE1" s="84"/>
@@ -13729,10 +13745,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="83"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -14115,36 +14131,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="41"/>
       <c r="AD1" s="41"/>
       <c r="AE1" s="41"/>
@@ -14191,10 +14207,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="40"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -14704,36 +14720,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="82"/>
       <c r="AD1" s="82"/>
       <c r="AE1" s="82"/>
@@ -14780,10 +14796,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -15135,19 +15151,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15205,19 +15221,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15276,19 +15292,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15357,19 +15373,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15438,19 +15454,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:6" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:6" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15518,19 +15534,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -15592,21 +15608,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
+      <c r="A1" s="119" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
     </row>
     <row r="2" spans="1:5" ht="18">
-      <c r="D2" s="109"/>
+      <c r="D2" s="117"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="116"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="108"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="116"/>
     </row>
     <row r="4" spans="1:5" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
@@ -15630,13 +15646,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>148</v>
+        <v>62</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="E5" s="67" t="s">
         <v>191</v>
@@ -15653,6 +15669,80 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="27.75" customHeight="1">
+      <c r="A1" s="119" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+    </row>
+    <row r="2" spans="1:5" ht="18">
+      <c r="D2" s="109"/>
+    </row>
+    <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="108"/>
+    </row>
+    <row r="4" spans="1:5" s="31" customFormat="1">
+      <c r="A4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="113" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15">
+      <c r="A5" s="10">
+        <v>1</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>191</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
@@ -15706,36 +15796,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="44"/>
       <c r="AD1" s="44"/>
       <c r="AE1" s="44"/>
@@ -15782,10 +15872,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="43"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -16294,36 +16384,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="46"/>
       <c r="AD1" s="46"/>
       <c r="AE1" s="46"/>
@@ -16370,10 +16460,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="45"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -16882,36 +16972,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="48"/>
       <c r="AD1" s="48"/>
       <c r="AE1" s="48"/>
@@ -16958,10 +17048,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="47"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -17470,36 +17560,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -17546,10 +17636,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -18058,36 +18148,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="50"/>
       <c r="AE1" s="50"/>
@@ -18134,10 +18224,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="49"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -18646,36 +18736,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="119"/>
+      <c r="V1" s="119"/>
+      <c r="W1" s="119"/>
+      <c r="X1" s="119"/>
+      <c r="Y1" s="119"/>
+      <c r="Z1" s="119"/>
+      <c r="AA1" s="119"/>
+      <c r="AB1" s="119"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -18722,10 +18812,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="116"/>
+      <c r="A3" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="118"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
Subcontract Function And Locators Changes Fixes
Subcontract Function And Locators Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="21" activeTab="21"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="30" activeTab="32"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2360" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="233">
   <si>
     <t>GST Sales</t>
   </si>
@@ -300,9 +300,6 @@
   </si>
   <si>
     <t>9620</t>
-  </si>
-  <si>
-    <t>78104</t>
   </si>
   <si>
     <t>PROD 100</t>
@@ -704,12 +701,6 @@
     <t>SORD-2526-00266</t>
   </si>
   <si>
-    <t>PROC- 5140</t>
-  </si>
-  <si>
-    <t>PROC- 7766</t>
-  </si>
-  <si>
     <t>99775</t>
   </si>
   <si>
@@ -752,25 +743,37 @@
     <t>99767.5</t>
   </si>
   <si>
-    <t>95801</t>
-  </si>
-  <si>
     <t>95786</t>
   </si>
   <si>
-    <t>95731</t>
+    <t>95641</t>
   </si>
   <si>
-    <t>95716</t>
+    <t>30</t>
   </si>
   <si>
-    <t>95686</t>
+    <t>PROC- 0226</t>
   </si>
   <si>
-    <t>95671</t>
+    <t>PROC- 1797</t>
   </si>
   <si>
-    <t>95641</t>
+    <t>PROC- 5304</t>
+  </si>
+  <si>
+    <t>PROC- 6708</t>
+  </si>
+  <si>
+    <t>PROC- 9688</t>
+  </si>
+  <si>
+    <t>PROC- 8659</t>
+  </si>
+  <si>
+    <t>PROC- 1431</t>
+  </si>
+  <si>
+    <t>PROC- 1925</t>
   </si>
 </sst>
 </file>
@@ -1995,13 +1998,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -2099,17 +2102,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>-15</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29">
         <v>87850</v>
@@ -2228,17 +2231,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9490</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -2597,7 +2600,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -2683,17 +2686,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9775</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -2721,7 +2724,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -2807,17 +2810,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9890</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="7"/>
       <c r="AL6" s="59"/>
@@ -3147,10 +3150,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -3159,13 +3162,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -3263,17 +3266,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>782</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -3610,10 +3613,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -3622,13 +3625,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -3726,17 +3729,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -3785,7 +3788,7 @@
     </row>
     <row r="9" spans="1:39">
       <c r="C9" s="89" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D9" s="23"/>
       <c r="E9" s="23"/>
@@ -3802,7 +3805,7 @@
     </row>
     <row r="10" spans="1:39">
       <c r="C10" s="90" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D10" s="90" t="s">
         <v>6</v>
@@ -3811,19 +3814,19 @@
         <v>7</v>
       </c>
       <c r="F10" s="90" t="s">
+        <v>86</v>
+      </c>
+      <c r="G10" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="G10" s="90" t="s">
+      <c r="H10" s="90" t="s">
         <v>88</v>
       </c>
-      <c r="H10" s="90" t="s">
+      <c r="I10" s="90" t="s">
         <v>89</v>
       </c>
-      <c r="I10" s="90" t="s">
+      <c r="J10" s="90" t="s">
         <v>90</v>
-      </c>
-      <c r="J10" s="90" t="s">
-        <v>91</v>
       </c>
       <c r="K10" s="90" t="s">
         <v>26</v>
@@ -3846,16 +3849,16 @@
         <v>1</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E11" s="10">
         <v>0</v>
       </c>
       <c r="F11" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>92</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="H11" s="10">
         <v>20</v>
@@ -3887,16 +3890,16 @@
         <v>2</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E12" s="10">
         <v>0</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H12" s="10"/>
       <c r="I12" s="10">
@@ -3928,7 +3931,7 @@
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I13" s="10">
         <v>21477.41</v>
@@ -4238,10 +4241,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -4250,13 +4253,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -4354,17 +4357,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -4701,10 +4704,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -4713,13 +4716,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -4817,17 +4820,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65248</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -4844,13 +4847,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="97" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="97" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -4948,17 +4951,17 @@
         <v>16</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AH6" s="34">
         <f>AG6-AF6</f>
         <v>99984</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="34">
         <f>AH6</f>
@@ -4974,13 +4977,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="97" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C7" s="10">
         <v>0</v>
       </c>
       <c r="D7" s="97" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>32</v>
@@ -5078,17 +5081,17 @@
         <v>17</v>
       </c>
       <c r="AG7" s="36" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AH7" s="34">
         <f t="shared" ref="AH7:AH14" si="20">AG7-AF7</f>
         <v>99983</v>
       </c>
       <c r="AI7" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ7" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ7" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK7" s="34">
         <f t="shared" ref="AK7:AK14" si="21">AH7</f>
@@ -5104,13 +5107,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
       </c>
       <c r="D8" s="97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>32</v>
@@ -5208,17 +5211,17 @@
         <v>18</v>
       </c>
       <c r="AG8" s="36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH8" s="34">
         <f t="shared" si="20"/>
         <v>99982</v>
       </c>
       <c r="AI8" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ8" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ8" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK8" s="34">
         <f t="shared" si="21"/>
@@ -5234,13 +5237,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="97" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
       </c>
       <c r="D9" s="97" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>32</v>
@@ -5338,17 +5341,17 @@
         <v>19</v>
       </c>
       <c r="AG9" s="36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AH9" s="34">
         <f t="shared" si="20"/>
         <v>99981</v>
       </c>
       <c r="AI9" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ9" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ9" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK9" s="34">
         <f t="shared" si="21"/>
@@ -5364,13 +5367,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="97" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
       </c>
       <c r="D10" s="97" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>32</v>
@@ -5468,17 +5471,17 @@
         <v>20</v>
       </c>
       <c r="AG10" s="36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AH10" s="34">
         <f t="shared" si="20"/>
         <v>99980</v>
       </c>
       <c r="AI10" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ10" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ10" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK10" s="34">
         <f t="shared" si="21"/>
@@ -5494,13 +5497,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="97" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" s="10">
         <v>0</v>
       </c>
       <c r="D11" s="97" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>32</v>
@@ -5598,17 +5601,17 @@
         <v>21</v>
       </c>
       <c r="AG11" s="36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AH11" s="34">
         <f t="shared" si="20"/>
         <v>99979</v>
       </c>
       <c r="AI11" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ11" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ11" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK11" s="34">
         <f t="shared" si="21"/>
@@ -5624,13 +5627,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="100" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" s="99">
         <v>0</v>
       </c>
       <c r="D12" s="100" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E12" s="99" t="s">
         <v>32</v>
@@ -5728,17 +5731,17 @@
         <v>22</v>
       </c>
       <c r="AG12" s="36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH12" s="102">
         <f t="shared" si="20"/>
         <v>99978</v>
       </c>
       <c r="AI12" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ12" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ12" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK12" s="102">
         <f t="shared" si="21"/>
@@ -5754,13 +5757,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="97" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C13" s="10">
         <v>0</v>
       </c>
       <c r="D13" s="97" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>32</v>
@@ -5858,17 +5861,17 @@
         <v>23</v>
       </c>
       <c r="AG13" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="34">
         <f t="shared" si="20"/>
         <v>99977</v>
       </c>
       <c r="AI13" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ13" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ13" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK13" s="34">
         <f t="shared" si="21"/>
@@ -5884,13 +5887,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="97" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C14" s="10">
         <v>0</v>
       </c>
       <c r="D14" s="97" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>32</v>
@@ -5988,17 +5991,17 @@
         <v>24</v>
       </c>
       <c r="AG14" s="36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AH14" s="34">
         <f t="shared" si="20"/>
         <v>99976</v>
       </c>
       <c r="AI14" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ14" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ14" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK14" s="34">
         <f t="shared" si="21"/>
@@ -7035,25 +7038,25 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="AN4" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="AO4" s="98" t="s">
         <v>107</v>
       </c>
-      <c r="AN4" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="AO4" s="98" t="s">
+      <c r="AP4" s="98" t="s">
         <v>108</v>
       </c>
-      <c r="AP4" s="98" t="s">
+      <c r="AQ4" s="98" t="s">
         <v>109</v>
-      </c>
-      <c r="AQ4" s="98" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="15">
@@ -7061,13 +7064,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -7164,18 +7167,18 @@
         <f>G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>231</v>
+      <c r="AG5" s="36" t="s">
+        <v>223</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
         <v>99656</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="33">
         <f>AH5</f>
@@ -7189,10 +7192,10 @@
         <v>66</v>
       </c>
       <c r="AN5" s="67" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AO5" s="29" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -7378,7 +7381,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -7527,7 +7530,7 @@
         <v>43</v>
       </c>
       <c r="AK4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AL4" s="58"/>
     </row>
@@ -7536,13 +7539,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -7640,17 +7643,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>99861</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="7">
         <f>IF($D$3=4,ROUND(((U5*W5)/2),2),0)</f>
@@ -7989,13 +7992,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -8093,17 +8096,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -8439,13 +8442,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -8543,17 +8546,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -8889,13 +8892,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -8993,17 +8996,17 @@
         <v>10</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80704</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -9339,7 +9342,7 @@
         <v>36</v>
       </c>
       <c r="AM4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:39" ht="15">
@@ -9347,13 +9350,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -9451,17 +9454,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>82574</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -9584,17 +9587,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9657.5</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -10047,10 +10050,10 @@
         <v>80704</v>
       </c>
       <c r="AI5" s="63" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -10494,10 +10497,10 @@
         <v>80704</v>
       </c>
       <c r="AI5" s="63" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -10837,13 +10840,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -10940,18 +10943,18 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>226</v>
+      <c r="AG5" s="36" t="s">
+        <v>222</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="66">
         <v>5</v>
@@ -11290,13 +11293,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -11394,17 +11397,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>63733</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="59"/>
     </row>
@@ -11845,17 +11848,17 @@
         <v>7.5</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9630</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="66" t="s">
         <v>72</v>
@@ -11867,13 +11870,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -11971,17 +11974,17 @@
         <v>15</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>78219</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="66" t="s">
         <v>71</v>
@@ -12277,10 +12280,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AL4" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:38" ht="15">
@@ -12405,10 +12408,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK5" s="72" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL5" s="72" t="s">
         <v>207</v>
-      </c>
-      <c r="AL5" s="72" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -12416,13 +12419,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -12533,10 +12536,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK6" s="66" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL6" s="66" t="s">
         <v>207</v>
-      </c>
-      <c r="AL6" s="66" t="s">
-        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -12828,10 +12831,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AL4" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:38" ht="15">
@@ -12956,10 +12959,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK5" s="72" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL5" s="72" t="s">
         <v>207</v>
-      </c>
-      <c r="AL5" s="72" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -12967,13 +12970,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -13084,10 +13087,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK6" s="66" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL6" s="66" t="s">
         <v>207</v>
-      </c>
-      <c r="AL6" s="66" t="s">
-        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -13379,10 +13382,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AL4" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:38" ht="15">
@@ -13498,16 +13501,16 @@
         <v>9612.5</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -13799,10 +13802,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AL4" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:38" ht="15">
@@ -13918,16 +13921,16 @@
         <v>-10</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -14219,10 +14222,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AL4" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:38" ht="15">
@@ -14338,16 +14341,16 @@
         <v>-5</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -14668,7 +14671,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -14754,17 +14757,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9645</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -14797,7 +14800,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -14883,17 +14886,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9950.6589999999997</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -15228,10 +15231,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -15240,13 +15243,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -15344,17 +15347,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>49586</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -15691,10 +15694,10 @@
         <v>43</v>
       </c>
       <c r="AK4" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AL4" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AM4" s="58"/>
     </row>
@@ -15703,13 +15706,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -15807,17 +15810,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -15889,7 +15892,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -15909,13 +15912,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>130</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>131</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15923,11 +15926,11 @@
       <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>209</v>
+      <c r="B5" t="s" s="29">
+        <v>232</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D5" s="10">
         <v>40</v>
@@ -15959,7 +15962,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -15979,13 +15982,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>130</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>131</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -15994,10 +15997,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D5" s="10">
         <v>30</v>
@@ -16034,7 +16037,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16057,46 +16060,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16104,16 +16107,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16147,10 +16150,10 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16187,7 +16190,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16210,46 +16213,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16257,16 +16260,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16300,10 +16303,10 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16342,7 +16345,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16365,46 +16368,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16412,16 +16415,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16455,10 +16458,10 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16497,7 +16500,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16520,46 +16523,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16567,16 +16570,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
+        <v>143</v>
+      </c>
+      <c r="C5" s="114" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="114" t="s">
-        <v>145</v>
-      </c>
       <c r="D5" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16607,13 +16610,13 @@
         <v>157.5</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16647,7 +16650,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16670,43 +16673,43 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15">
@@ -16714,16 +16717,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16754,10 +16757,10 @@
         <v>135</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
     </row>
   </sheetData>
@@ -16790,7 +16793,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -16813,46 +16816,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16860,16 +16863,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16903,10 +16906,10 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -17233,7 +17236,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -17319,17 +17322,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9745</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -17448,17 +17451,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9880</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -17530,7 +17533,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -17553,43 +17556,43 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>161</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O4" s="115" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15">
@@ -17597,16 +17600,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -17640,7 +17643,7 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
     </row>
   </sheetData>
@@ -17701,7 +17704,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -17787,7 +17790,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -17797,7 +17800,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -17831,34 +17834,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -17876,7 +17879,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -17891,25 +17894,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -17927,7 +17930,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -18055,7 +18058,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -18141,7 +18144,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -18151,7 +18154,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -18185,34 +18188,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -18230,7 +18233,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -18245,25 +18248,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -18281,7 +18284,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -18409,7 +18412,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -18495,7 +18498,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -18505,7 +18508,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -18539,34 +18542,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -18584,7 +18587,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -18599,25 +18602,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -18635,7 +18638,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -18763,7 +18766,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -18849,7 +18852,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -18859,7 +18862,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -18893,34 +18896,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -18938,7 +18941,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -18953,25 +18956,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -18989,7 +18992,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -19117,7 +19120,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -19203,7 +19206,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -19213,7 +19216,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -19247,34 +19250,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -19292,7 +19295,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -19307,25 +19310,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>224</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -19343,7 +19346,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -19471,7 +19474,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -19557,7 +19560,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -19567,7 +19570,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -19601,34 +19604,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -19646,7 +19649,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -19661,25 +19664,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -19697,7 +19700,7 @@
         <v>32</v>
       </c>
       <c r="M5" s="33">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="N5" s="22">
         <v>0.18</v>
@@ -19798,7 +19801,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -19821,49 +19824,49 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="115" t="s">
+      <c r="N4" s="115" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="115" t="s">
+        <v>90</v>
+      </c>
+      <c r="P4" s="115" t="s">
         <v>161</v>
       </c>
-      <c r="N4" s="115" t="s">
-        <v>166</v>
-      </c>
-      <c r="O4" s="115" t="s">
-        <v>91</v>
-      </c>
-      <c r="P4" s="115" t="s">
+      <c r="Q4" s="115" t="s">
         <v>162</v>
-      </c>
-      <c r="Q4" s="115" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15">
@@ -19871,16 +19874,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
@@ -19914,13 +19917,13 @@
         <v>32</v>
       </c>
       <c r="O5" s="123">
-        <v>88363222</v>
+        <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q5" s="10" t="s">
         <v>164</v>
-      </c>
-      <c r="Q5" s="10" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -19984,7 +19987,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="165" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -20070,7 +20073,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -20080,7 +20083,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -20114,34 +20117,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>131</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>156</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>157</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>158</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>159</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -20159,7 +20162,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -20174,25 +20177,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -20369,7 +20372,7 @@
     </row>
     <row r="2" spans="1:38" ht="18">
       <c r="A2" s="134" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B2" s="134"/>
       <c r="C2" s="134"/>
@@ -20413,7 +20416,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="140" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F3" s="141"/>
       <c r="G3" s="141"/>
@@ -20572,13 +20575,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" s="155">
         <v>0</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" s="155" t="s">
         <v>32</v>
@@ -20642,7 +20645,7 @@
         <v>11493.38</v>
       </c>
       <c r="V5" s="155" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="W5" s="156">
         <v>0.18</v>
@@ -20682,17 +20685,17 @@
         <v>10</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>99896</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29">
         <v>87850</v>
@@ -20707,16 +20710,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C6" s="155">
         <v>0</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E6" s="155" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F6" s="155" t="s">
         <v>32</v>
@@ -20777,7 +20780,7 @@
         <v>26656.080000000002</v>
       </c>
       <c r="V6" s="155" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="W6" s="156">
         <v>0.18</v>
@@ -20817,17 +20820,17 @@
         <v>3.3330000000000002</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>99966.667000000001</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -20855,7 +20858,7 @@
       <c r="O7" s="159"/>
       <c r="P7" s="161"/>
       <c r="Q7" s="161" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="R7" s="161"/>
       <c r="S7" s="161"/>
@@ -20866,7 +20869,7 @@
       <c r="X7" s="159"/>
       <c r="Y7" s="159"/>
       <c r="Z7" s="161" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="AA7" s="161"/>
       <c r="AB7" s="162">
@@ -20874,7 +20877,7 @@
         <v>45016.36</v>
       </c>
       <c r="AC7" s="161" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="AD7" s="162">
         <f>SUM(AD5:AD6)</f>
@@ -21324,17 +21327,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9717</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -21367,7 +21370,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -21453,17 +21456,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9865</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -21826,7 +21829,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -21912,17 +21915,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9795</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -21955,7 +21958,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -22041,17 +22044,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9900</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -22414,7 +22417,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -22500,17 +22503,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9703</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -22543,7 +22546,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -22629,17 +22632,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9852.5</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -23002,7 +23005,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -23088,17 +23091,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -23131,7 +23134,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -23217,17 +23220,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -23590,7 +23593,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -23676,17 +23679,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -23719,7 +23722,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -23805,17 +23808,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
Subcontract Function And Locator Changes Fixes
Subcontract Function And Locator Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="34" activeTab="39"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="22" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2470" uniqueCount="233">
   <si>
     <t>GST Sales</t>
   </si>
@@ -730,9 +730,6 @@
     <t>95786</t>
   </si>
   <si>
-    <t>95641</t>
-  </si>
-  <si>
     <t>SORD-2526-00764</t>
   </si>
   <si>
@@ -779,9 +776,6 @@
   </si>
   <si>
     <t>40</t>
-  </si>
-  <si>
-    <t>93041</t>
   </si>
   <si>
     <t>93026</t>
@@ -2126,7 +2120,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -2255,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -7191,8 +7185,8 @@
         <f>G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>234</v>
+      <c r="AG5" s="36" t="s">
+        <v>232</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
@@ -12703,7 +12697,7 @@
       <c r="B3" s="169"/>
       <c r="C3" s="70"/>
       <c r="D3" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>1</v>
@@ -12945,15 +12939,15 @@
       </c>
       <c r="Z5" s="34">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>0</v>
+        <v>378</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>0</v>
+        <v>378</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>2100</v>
+        <v>2478</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
@@ -13073,15 +13067,15 @@
       </c>
       <c r="Z6" s="34">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>600</v>
+        <v>708</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
@@ -15378,7 +15372,7 @@
         <v>49586</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>175</v>
@@ -15834,14 +15828,14 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>175</v>
@@ -15951,7 +15945,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>130</v>
@@ -16021,7 +16015,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>129</v>
@@ -16177,7 +16171,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16332,7 +16326,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16485,7 +16479,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16793,7 +16787,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="166" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16948,7 +16942,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -17691,7 +17685,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17846,7 +17840,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -18706,7 +18700,7 @@
         <v>129</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>162</v>
@@ -19060,7 +19054,7 @@
         <v>129</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>162</v>
@@ -19414,7 +19408,7 @@
         <v>129</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>162</v>
@@ -19768,7 +19762,7 @@
         <v>129</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>162</v>
@@ -20698,7 +20692,7 @@
         <v>123</v>
       </c>
       <c r="C5" t="s" s="29">
-        <v>57</v>
+        <v>141</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>126</v>
@@ -20710,7 +20704,7 @@
         <v>129</v>
       </c>
       <c r="G5" t="s" s="29">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" t="s" s="29">
         <v>162</v>
@@ -21051,7 +21045,7 @@
       <c r="B5" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="C5" t="s" s="29">
+      <c r="C5" s="29" t="s">
         <v>141</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -21060,13 +21054,13 @@
       <c r="E5" s="67" t="s">
         <v>136</v>
       </c>
-      <c r="F5" t="s" s="29">
+      <c r="F5" s="29" t="s">
         <v>129</v>
       </c>
-      <c r="G5" t="s" s="29">
-        <v>232</v>
-      </c>
-      <c r="H5" t="s" s="29">
+      <c r="G5" s="29" t="s">
+        <v>231</v>
+      </c>
+      <c r="H5" s="29" t="s">
         <v>162</v>
       </c>
       <c r="I5" s="10">
@@ -21081,7 +21075,7 @@
         <f>I5*G5</f>
         <v>625</v>
       </c>
-      <c r="L5" t="s" s="29">
+      <c r="L5" s="29" t="s">
         <v>32</v>
       </c>
       <c r="M5" s="33">

</xml_diff>

<commit_message>
Sales Invoice Function and Sales Invoice Locators Fixes Changes
Sales Invoice Function and Sales Invoice Locators Fixes Changes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2479" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="251">
   <si>
     <t>GST Sales</t>
   </si>
@@ -813,6 +813,27 @@
   </si>
   <si>
     <t>99710</t>
+  </si>
+  <si>
+    <t>90931</t>
+  </si>
+  <si>
+    <t>90916</t>
+  </si>
+  <si>
+    <t>90901</t>
+  </si>
+  <si>
+    <t>90886</t>
+  </si>
+  <si>
+    <t>90871</t>
+  </si>
+  <si>
+    <t>90856</t>
+  </si>
+  <si>
+    <t>99830</t>
   </si>
 </sst>
 </file>
@@ -1780,43 +1801,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="14.0"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2368,43 +2389,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2942,44 +2963,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3405,44 +3426,44 @@
   <dimension ref="A1:AM13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="18.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4033,44 +4054,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4496,44 +4517,44 @@
   <dimension ref="A1:AM36"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -6826,48 +6847,48 @@
   <dimension ref="A1:AQ6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="36" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="41" width="14.140625" style="29" customWidth="1"/>
-    <col min="42" max="42" width="15" style="29" customWidth="1"/>
-    <col min="43" max="43" width="16.5703125" style="29" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="36.0"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="41" customWidth="true" style="29" width="14.140625"/>
+    <col min="42" max="42" customWidth="true" style="29" width="15.0"/>
+    <col min="43" max="43" customWidth="true" style="29" width="16.5703125"/>
+    <col min="44" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
@@ -7234,8 +7255,8 @@
         <f>G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" s="36" t="s">
-        <v>241</v>
+      <c r="AG5" t="s" s="36">
+        <v>249</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
@@ -7255,14 +7276,14 @@
         <f>AK5+G5</f>
         <v>99671</v>
       </c>
-      <c r="AM5" s="28" t="s">
+      <c r="AM5" t="s" s="28">
         <v>66</v>
       </c>
       <c r="AN5" s="67" t="s">
         <v>176</v>
       </c>
-      <c r="AO5" s="29" t="s">
-        <v>120</v>
+      <c r="AO5" t="s" s="29">
+        <v>250</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -7323,43 +7344,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.5703125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="21.28515625" style="29" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="34.5703125"/>
+    <col min="8" max="8" customWidth="true" style="29" width="21.28515625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -7778,43 +7799,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8228,43 +8249,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8678,43 +8699,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9128,44 +9149,44 @@
   <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -9728,43 +9749,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10175,43 +10196,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10622,43 +10643,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -11081,42 +11102,42 @@
   <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.42578125" style="29" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="15.42578125"/>
+    <col min="38" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
@@ -11528,43 +11549,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12073,43 +12094,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12624,43 +12645,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13175,43 +13196,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13595,43 +13616,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14015,43 +14036,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="11.7109375" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="11.7109375"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14435,43 +14456,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -15023,44 +15044,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15486,44 +15507,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15949,12 +15970,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16019,12 +16040,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16089,17 +16110,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16244,17 +16265,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16399,15 +16420,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="14.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="14.85546875"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16552,15 +16573,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16705,17 +16726,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16860,17 +16881,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17015,43 +17036,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -17603,17 +17624,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17758,17 +17779,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17913,12 +17934,12 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18051,17 +18072,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18206,17 +18227,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18361,14 +18382,14 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11" style="29" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.0"/>
+    <col min="11" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18501,45 +18522,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -18855,45 +18876,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19209,45 +19230,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19563,45 +19584,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19917,43 +19938,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -20505,45 +20526,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -20859,45 +20880,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -21213,18 +21234,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21372,13 +21393,13 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
+    <col min="3" max="3" customWidth="true" style="29" width="14.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="15.5703125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="7" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
@@ -21463,45 +21484,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -21817,40 +21838,40 @@
   <dimension ref="A1:AL8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="137" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="137" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="137" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="137" customWidth="1"/>
-    <col min="5" max="5" width="10" style="137" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="137" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="137" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="137" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="137" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="137" customWidth="1"/>
-    <col min="12" max="12" width="8" style="137" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="137" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="137" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="137" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="137" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="137" customWidth="1"/>
-    <col min="18" max="18" width="9" style="137" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="137" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="137" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="137" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" style="137" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="137" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="137" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="137" customWidth="1"/>
-    <col min="27" max="27" width="12" style="137" customWidth="1"/>
-    <col min="28" max="28" width="12.28515625" style="137" customWidth="1"/>
-    <col min="29" max="29" width="14.7109375" style="137" customWidth="1"/>
-    <col min="30" max="30" width="12.28515625" style="163" customWidth="1"/>
-    <col min="31" max="31" width="13.5703125" style="163" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.5703125" style="163" customWidth="1"/>
-    <col min="33" max="33" width="15.7109375" style="136" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.5703125" style="137" customWidth="1"/>
-    <col min="35" max="35" width="12.7109375" style="137" customWidth="1"/>
-    <col min="36" max="16384" width="9.140625" style="137"/>
+    <col min="1" max="1" customWidth="true" style="137" width="5.7109375"/>
+    <col min="2" max="2" customWidth="true" style="137" width="28.85546875"/>
+    <col min="3" max="3" customWidth="true" style="137" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="137" width="28.85546875"/>
+    <col min="5" max="5" customWidth="true" style="137" width="10.0"/>
+    <col min="6" max="6" customWidth="true" style="137" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="137" width="14.7109375"/>
+    <col min="8" max="8" customWidth="true" style="137" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="137" width="13.5703125"/>
+    <col min="10" max="11" customWidth="true" style="137" width="8.140625"/>
+    <col min="12" max="12" customWidth="true" style="137" width="8.0"/>
+    <col min="13" max="13" customWidth="true" style="137" width="13.85546875"/>
+    <col min="14" max="14" customWidth="true" style="137" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="137" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="137" width="14.7109375"/>
+    <col min="17" max="17" customWidth="true" style="137" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="137" width="9.0"/>
+    <col min="19" max="19" customWidth="true" style="137" width="10.85546875"/>
+    <col min="20" max="20" customWidth="true" style="137" width="17.85546875"/>
+    <col min="21" max="21" customWidth="true" style="137" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="137" width="11.5703125"/>
+    <col min="23" max="23" customWidth="true" style="137" width="9.28515625"/>
+    <col min="24" max="25" customWidth="true" style="137" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="137" width="11.28515625"/>
+    <col min="27" max="27" customWidth="true" style="137" width="12.0"/>
+    <col min="28" max="28" customWidth="true" style="137" width="12.28515625"/>
+    <col min="29" max="29" customWidth="true" style="137" width="14.7109375"/>
+    <col min="30" max="30" customWidth="true" style="163" width="12.28515625"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="163" width="13.5703125"/>
+    <col min="32" max="32" customWidth="true" style="163" width="13.5703125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="136" width="15.7109375"/>
+    <col min="34" max="34" customWidth="true" style="137" width="13.5703125"/>
+    <col min="35" max="35" customWidth="true" style="137" width="12.7109375"/>
+    <col min="36" max="16384" style="137" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -22457,43 +22478,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23045,43 +23066,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23633,43 +23654,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24221,43 +24242,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">

</xml_diff>

<commit_message>
Subcontract Test And Subcontract Function fixes Changes
Subcontract Test And Subcontract Function fixes Changes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="44" activeTab="47"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="36" activeTab="33"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2480" uniqueCount="245">
   <si>
     <t>GST Sales</t>
   </si>
@@ -441,9 +441,6 @@
   </si>
   <si>
     <t>105596</t>
-  </si>
-  <si>
-    <t>100001867</t>
   </si>
   <si>
     <t>Process</t>
@@ -806,34 +803,19 @@
     <t>PROC- 5049</t>
   </si>
   <si>
-    <t>91316</t>
-  </si>
-  <si>
     <t>99725</t>
   </si>
   <si>
     <t>99710</t>
   </si>
   <si>
-    <t>90931</t>
-  </si>
-  <si>
-    <t>90916</t>
-  </si>
-  <si>
-    <t>90901</t>
-  </si>
-  <si>
-    <t>90886</t>
-  </si>
-  <si>
-    <t>90871</t>
-  </si>
-  <si>
     <t>90856</t>
   </si>
   <si>
     <t>99830</t>
+  </si>
+  <si>
+    <t>PROC- 0744</t>
   </si>
 </sst>
 </file>
@@ -2086,13 +2068,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -2190,17 +2172,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>-15</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29">
         <v>87850</v>
@@ -2319,17 +2301,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9490</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -2688,7 +2670,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -2774,17 +2756,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9775</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -2812,7 +2794,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -2898,17 +2880,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9890</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="7"/>
       <c r="AL6" s="59"/>
@@ -3361,10 +3343,10 @@
         <v>782</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -3713,13 +3695,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -3817,17 +3799,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -3937,7 +3919,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E11" s="10">
         <v>0</v>
@@ -3978,7 +3960,7 @@
         <v>2</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E12" s="10">
         <v>0</v>
@@ -4445,17 +4427,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -4804,13 +4786,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -4915,10 +4897,10 @@
         <v>65248</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -5046,10 +5028,10 @@
         <v>99984</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="34">
         <f>AH6</f>
@@ -5176,10 +5158,10 @@
         <v>99983</v>
       </c>
       <c r="AI7" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ7" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ7" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK7" s="34">
         <f t="shared" ref="AK7:AK14" si="21">AH7</f>
@@ -5306,10 +5288,10 @@
         <v>99982</v>
       </c>
       <c r="AI8" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ8" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ8" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK8" s="34">
         <f t="shared" si="21"/>
@@ -5436,10 +5418,10 @@
         <v>99981</v>
       </c>
       <c r="AI9" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ9" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ9" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK9" s="34">
         <f t="shared" si="21"/>
@@ -5566,10 +5548,10 @@
         <v>99980</v>
       </c>
       <c r="AI10" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ10" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ10" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK10" s="34">
         <f t="shared" si="21"/>
@@ -5696,10 +5678,10 @@
         <v>99979</v>
       </c>
       <c r="AI11" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ11" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ11" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK11" s="34">
         <f t="shared" si="21"/>
@@ -5826,10 +5808,10 @@
         <v>99978</v>
       </c>
       <c r="AI12" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ12" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ12" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK12" s="102">
         <f t="shared" si="21"/>
@@ -5956,10 +5938,10 @@
         <v>99977</v>
       </c>
       <c r="AI13" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ13" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ13" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK13" s="34">
         <f t="shared" si="21"/>
@@ -6086,10 +6068,10 @@
         <v>99976</v>
       </c>
       <c r="AI14" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ14" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ14" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK14" s="34">
         <f t="shared" si="21"/>
@@ -7152,13 +7134,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -7255,18 +7237,18 @@
         <f>G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" t="s" s="36">
-        <v>249</v>
+      <c r="AG5" s="36" t="s">
+        <v>242</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
         <v>99656</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="33">
         <f>AH5</f>
@@ -7276,14 +7258,14 @@
         <f>AK5+G5</f>
         <v>99671</v>
       </c>
-      <c r="AM5" t="s" s="28">
+      <c r="AM5" s="28" t="s">
         <v>66</v>
       </c>
       <c r="AN5" s="67" t="s">
-        <v>176</v>
-      </c>
-      <c r="AO5" t="s" s="29">
-        <v>250</v>
+        <v>175</v>
+      </c>
+      <c r="AO5" s="29" t="s">
+        <v>243</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -7469,7 +7451,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -7618,7 +7600,7 @@
         <v>43</v>
       </c>
       <c r="AK4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AL4" s="58"/>
     </row>
@@ -7627,13 +7609,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -7731,17 +7713,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>99861</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="7">
         <f>IF($D$3=4,ROUND(((U5*W5)/2),2),0)</f>
@@ -8080,13 +8062,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -8184,17 +8166,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -8530,13 +8512,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -8634,17 +8616,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -8980,13 +8962,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -9084,17 +9066,17 @@
         <v>10</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80704</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -9438,13 +9420,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -9542,17 +9524,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>82574</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -9675,17 +9657,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9657.5</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -10138,10 +10120,10 @@
         <v>80704</v>
       </c>
       <c r="AI5" s="63" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -10588,7 +10570,7 @@
         <v>75</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AK5" s="7"/>
       <c r="AL5" s="59"/>
@@ -10928,13 +10910,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -11032,17 +11014,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="66">
         <v>5</v>
@@ -11381,13 +11363,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -11485,17 +11467,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>63733</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="59"/>
     </row>
@@ -11936,17 +11918,17 @@
         <v>7.5</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9630</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="66" t="s">
         <v>72</v>
@@ -11958,13 +11940,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -12062,17 +12044,17 @@
         <v>15</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>78219</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="66" t="s">
         <v>71</v>
@@ -12496,10 +12478,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK5" s="72" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL5" s="72" t="s">
         <v>200</v>
-      </c>
-      <c r="AL5" s="72" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -12507,13 +12489,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -12624,10 +12606,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK6" s="66" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL6" s="66" t="s">
         <v>200</v>
-      </c>
-      <c r="AL6" s="66" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -13047,10 +13029,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK5" s="72" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL5" s="72" t="s">
         <v>200</v>
-      </c>
-      <c r="AL5" s="72" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -13058,13 +13040,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -13175,10 +13157,10 @@
         <v>4010101001</v>
       </c>
       <c r="AK6" s="66" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL6" s="66" t="s">
         <v>200</v>
-      </c>
-      <c r="AL6" s="66" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -13589,13 +13571,13 @@
         <v>9612.5</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AL5" s="72" t="s">
         <v>77</v>
@@ -14009,13 +13991,13 @@
         <v>-10</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AL5" s="72" t="s">
         <v>77</v>
@@ -14429,13 +14411,13 @@
         <v>-5</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
-      </c>
       <c r="AK5" s="72" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AL5" s="72" t="s">
         <v>77</v>
@@ -14759,7 +14741,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -14845,17 +14827,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9645</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -14888,7 +14870,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -14974,17 +14956,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9950.6589999999997</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -15331,13 +15313,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -15435,17 +15417,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>49586</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -15794,13 +15776,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -15898,17 +15880,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
@@ -15980,7 +15962,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16000,13 +15982,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>126</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>127</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -16014,11 +15996,11 @@
       <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>219</v>
+      <c r="B5" t="s" s="29">
+        <v>244</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" s="10">
         <v>40</v>
@@ -16050,7 +16032,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16070,13 +16052,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>126</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>127</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -16085,10 +16067,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D5" s="10">
         <v>30</v>
@@ -16125,7 +16107,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16148,46 +16130,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16195,16 +16177,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16241,7 +16223,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16280,7 +16262,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16303,46 +16285,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16350,16 +16332,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16396,7 +16378,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16433,7 +16415,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16456,46 +16438,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16503,16 +16485,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16549,7 +16531,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16586,7 +16568,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16609,46 +16591,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16656,16 +16638,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16702,7 +16684,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16741,7 +16723,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16764,46 +16746,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16811,16 +16793,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -16857,7 +16839,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="166" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16896,7 +16878,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -16919,46 +16901,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -16966,16 +16948,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" s="114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -17012,7 +16994,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -17339,7 +17321,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -17425,17 +17407,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9745</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -17554,17 +17536,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9880</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -17639,7 +17621,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -17662,46 +17644,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -17709,16 +17691,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="114" t="s">
         <v>139</v>
       </c>
-      <c r="C5" s="114" t="s">
-        <v>140</v>
-      </c>
       <c r="D5" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -17749,13 +17731,13 @@
         <v>157.5</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="O5" s="123">
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17794,7 +17776,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -17817,46 +17799,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -17864,16 +17846,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="114" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="114" t="s">
         <v>139</v>
       </c>
-      <c r="C5" s="114" t="s">
-        <v>140</v>
-      </c>
       <c r="D5" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -17904,13 +17886,13 @@
         <v>157.5</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="O5" s="123">
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17944,7 +17926,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -17967,40 +17949,40 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
@@ -18011,16 +17993,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -18051,7 +18033,7 @@
         <v>135</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="O5" s="123">
         <v>88363221</v>
@@ -18087,7 +18069,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -18110,46 +18092,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -18157,16 +18139,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -18203,7 +18185,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -18242,7 +18224,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -18265,46 +18247,46 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
@@ -18312,16 +18294,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -18358,7 +18340,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -18394,7 +18376,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -18417,40 +18399,40 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
@@ -18461,16 +18443,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -18565,7 +18547,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -18651,7 +18633,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -18661,7 +18643,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -18695,34 +18677,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -18740,7 +18722,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -18755,25 +18737,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -18919,7 +18901,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -19005,7 +18987,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -19015,7 +18997,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -19049,34 +19031,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -19094,7 +19076,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -19109,25 +19091,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -19273,7 +19255,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -19359,7 +19341,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -19369,7 +19351,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -19403,34 +19385,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -19448,7 +19430,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -19463,25 +19445,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>54</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -19627,7 +19609,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -19713,7 +19695,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -19723,7 +19705,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -19757,34 +19739,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -19802,7 +19784,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -19817,25 +19799,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -20327,17 +20309,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9717</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -20370,7 +20352,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -20456,17 +20438,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9865</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -20569,7 +20551,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -20655,7 +20637,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -20665,7 +20647,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -20699,34 +20681,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -20744,7 +20726,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -20759,25 +20741,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -20923,7 +20905,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -21009,7 +20991,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -21019,7 +21001,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -21053,34 +21035,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -21098,7 +21080,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -21113,25 +21095,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -21250,7 +21232,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -21273,49 +21255,49 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="115" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
+      <c r="L4" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="L4" s="115" t="s">
+      <c r="M4" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="M4" s="115" t="s">
-        <v>154</v>
-      </c>
       <c r="N4" s="115" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O4" s="115" t="s">
         <v>89</v>
       </c>
       <c r="P4" s="115" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q4" s="115" t="s">
         <v>155</v>
-      </c>
-      <c r="Q4" s="115" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15">
@@ -21323,16 +21305,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
@@ -21369,10 +21351,10 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q5" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="Q5" s="10" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -21404,7 +21386,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -21415,54 +21397,54 @@
     </row>
     <row r="3" spans="1:8" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="172" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
       <c r="D3" s="172"/>
       <c r="E3" s="173" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F3" s="173"/>
     </row>
     <row r="4" spans="1:8" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>233</v>
-      </c>
       <c r="D4" s="11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E4" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>229</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15">
       <c r="A5" s="122" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D5" s="10">
         <v>11</v>
       </c>
       <c r="E5" s="122" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F5" s="114" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -21527,7 +21509,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
       <c r="A1" s="171" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B1" s="171"/>
       <c r="C1" s="171"/>
@@ -21613,7 +21595,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -21623,7 +21605,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -21657,34 +21639,34 @@
         <v>6</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F4" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="126" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>127</v>
-      </c>
       <c r="H4" s="126" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="115" t="s">
+      <c r="J4" s="115" t="s">
         <v>150</v>
       </c>
-      <c r="J4" s="115" t="s">
+      <c r="K4" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K4" s="115" t="s">
-        <v>152</v>
-      </c>
       <c r="L4" s="127" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>25</v>
@@ -21702,7 +21684,7 @@
         <v>29</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S4" s="17" t="s">
         <v>30</v>
@@ -21717,25 +21699,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
@@ -21912,7 +21894,7 @@
     </row>
     <row r="2" spans="1:38" ht="18">
       <c r="A2" s="134" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B2" s="134"/>
       <c r="C2" s="134"/>
@@ -21956,7 +21938,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="140" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F3" s="141"/>
       <c r="G3" s="141"/>
@@ -22185,7 +22167,7 @@
         <v>11493.38</v>
       </c>
       <c r="V5" s="155" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="W5" s="156">
         <v>0.18</v>
@@ -22225,17 +22207,17 @@
         <v>10</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>99896</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29">
         <v>87850</v>
@@ -22250,16 +22232,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C6" s="155">
         <v>0</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E6" s="155" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F6" s="155" t="s">
         <v>32</v>
@@ -22320,7 +22302,7 @@
         <v>26656.080000000002</v>
       </c>
       <c r="V6" s="155" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="W6" s="156">
         <v>0.18</v>
@@ -22360,17 +22342,17 @@
         <v>3.3330000000000002</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>99966.667000000001</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -22398,7 +22380,7 @@
       <c r="O7" s="159"/>
       <c r="P7" s="161"/>
       <c r="Q7" s="161" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="R7" s="161"/>
       <c r="S7" s="161"/>
@@ -22409,7 +22391,7 @@
       <c r="X7" s="159"/>
       <c r="Y7" s="159"/>
       <c r="Z7" s="161" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AA7" s="161"/>
       <c r="AB7" s="162">
@@ -22417,7 +22399,7 @@
         <v>45016.36</v>
       </c>
       <c r="AC7" s="161" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AD7" s="162">
         <f>SUM(AD5:AD6)</f>
@@ -22781,7 +22763,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -22867,17 +22849,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9795</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -22910,7 +22892,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -22996,17 +22978,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9900</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -23369,7 +23351,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -23455,17 +23437,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9703</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -23498,7 +23480,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -23584,17 +23566,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9852.5</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -23957,7 +23939,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -24043,17 +24025,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -24086,7 +24068,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -24172,17 +24154,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>
@@ -24545,7 +24527,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
@@ -24631,17 +24613,17 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
         <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK5" s="29" t="s">
         <v>46</v>
@@ -24674,7 +24656,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
@@ -24760,17 +24742,17 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
         <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="AJ6" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="AK6" s="29" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
New Subcontract Order Scenarios Added And Sales Invoice Changes Fixes
New Subcontract Order Scenarios Added And Sales Invoice Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="51" activeTab="57"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="47" activeTab="51"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -58,13 +58,11 @@
     <sheet name="ProcCalculationUTGSTUnreg" sheetId="55" r:id="rId49"/>
     <sheet name="ProcCalculationInterstateUnreg" sheetId="54" r:id="rId50"/>
     <sheet name="ProcCalculationLocalReg" sheetId="51" r:id="rId51"/>
-    <sheet name="DirectSCO" sheetId="39" r:id="rId52"/>
-    <sheet name="SourceSFCode" sheetId="67" r:id="rId53"/>
-    <sheet name="SCOCharges" sheetId="57" r:id="rId54"/>
-    <sheet name="SOtoSIDomestic" sheetId="61" r:id="rId55"/>
-    <sheet name="BRSPMI" sheetId="68" r:id="rId56"/>
-    <sheet name="BRSPSIE" sheetId="69" r:id="rId57"/>
-    <sheet name="BRSPSI" sheetId="70" r:id="rId58"/>
+    <sheet name="DirectSCOWithQC" sheetId="68" r:id="rId52"/>
+    <sheet name="DirectSCO" sheetId="39" r:id="rId53"/>
+    <sheet name="SourceSFCode" sheetId="67" r:id="rId54"/>
+    <sheet name="SCOCharges" sheetId="57" r:id="rId55"/>
+    <sheet name="SOtoSIDomestic" sheetId="61" r:id="rId56"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -84,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2638" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2503" uniqueCount="246">
   <si>
     <t>GST Sales</t>
   </si>
@@ -686,6 +684,9 @@
     <t>SORD-2526-00077</t>
   </si>
   <si>
+    <t>SORD-2526-00266</t>
+  </si>
+  <si>
     <t>99775</t>
   </si>
   <si>
@@ -800,12 +801,6 @@
     <t>PROC- 5049</t>
   </si>
   <si>
-    <t>99725</t>
-  </si>
-  <si>
-    <t>99710</t>
-  </si>
-  <si>
     <t>90856</t>
   </si>
   <si>
@@ -815,16 +810,16 @@
     <t>PROC- 0744</t>
   </si>
   <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>FG70001-QC-LOT</t>
+  </si>
+  <si>
     <t>SORD-2526-01270</t>
   </si>
   <si>
-    <t>91006</t>
-  </si>
-  <si>
-    <t>93816</t>
-  </si>
-  <si>
-    <t>91021</t>
+    <t>99175</t>
   </si>
 </sst>
 </file>
@@ -2187,11 +2182,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>93996</v>
+        <v>-15</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -2316,11 +2311,11 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99587.5</v>
+        <v>9490</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -2689,14 +2684,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -2704,7 +2699,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -2712,7 +2707,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -2728,7 +2723,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -2746,22 +2741,22 @@
       </c>
       <c r="Z5" s="9">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1176</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -2775,7 +2770,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99985</v>
+        <v>9775</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -2813,14 +2808,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -2828,7 +2823,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -2836,7 +2831,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -2852,7 +2847,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -2870,22 +2865,22 @@
       </c>
       <c r="Z6" s="9">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>896</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -2899,7 +2894,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99995</v>
+        <v>9890</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -3355,7 +3350,7 @@
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>105581</v>
+        <v>782</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -3365,11 +3360,11 @@
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>105581</v>
+        <v>782</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>105596</v>
+        <v>797</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -3818,7 +3813,7 @@
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>99641</v>
+        <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -3828,11 +3823,11 @@
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>99641</v>
+        <v>65983</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>99656</v>
+        <v>65998</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -4446,7 +4441,7 @@
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>99985</v>
+        <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -4456,11 +4451,11 @@
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>99985</v>
+        <v>65983</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>100000</v>
+        <v>65998</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -4909,7 +4904,7 @@
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>62703</v>
+        <v>65248</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -4919,11 +4914,11 @@
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>62703</v>
+        <v>65248</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>62718</v>
+        <v>65263</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -5040,7 +5035,7 @@
       </c>
       <c r="AH6" s="34">
         <f>AG6-AF6</f>
-        <v>99920</v>
+        <v>99984</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -5050,11 +5045,11 @@
       </c>
       <c r="AK6" s="34">
         <f>AH6</f>
-        <v>99920</v>
+        <v>99984</v>
       </c>
       <c r="AL6" s="34">
         <f>AK6+G6</f>
-        <v>99936</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="7" spans="1:39">
@@ -5170,7 +5165,7 @@
       </c>
       <c r="AH7" s="34">
         <f t="shared" ref="AH7:AH14" si="20">AG7-AF7</f>
-        <v>99915</v>
+        <v>99983</v>
       </c>
       <c r="AI7" s="10" t="s">
         <v>172</v>
@@ -5180,11 +5175,11 @@
       </c>
       <c r="AK7" s="34">
         <f t="shared" ref="AK7:AK14" si="21">AH7</f>
-        <v>99915</v>
+        <v>99983</v>
       </c>
       <c r="AL7" s="34">
         <f t="shared" ref="AL7:AL14" si="22">AK7+G7</f>
-        <v>99932</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="8" spans="1:39">
@@ -5300,7 +5295,7 @@
       </c>
       <c r="AH8" s="34">
         <f t="shared" si="20"/>
-        <v>99910</v>
+        <v>99982</v>
       </c>
       <c r="AI8" s="10" t="s">
         <v>172</v>
@@ -5310,11 +5305,11 @@
       </c>
       <c r="AK8" s="34">
         <f t="shared" si="21"/>
-        <v>99910</v>
+        <v>99982</v>
       </c>
       <c r="AL8" s="34">
         <f t="shared" si="22"/>
-        <v>99928</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="9" spans="1:39">
@@ -5430,7 +5425,7 @@
       </c>
       <c r="AH9" s="34">
         <f t="shared" si="20"/>
-        <v>99905</v>
+        <v>99981</v>
       </c>
       <c r="AI9" s="10" t="s">
         <v>172</v>
@@ -5440,11 +5435,11 @@
       </c>
       <c r="AK9" s="34">
         <f t="shared" si="21"/>
-        <v>99905</v>
+        <v>99981</v>
       </c>
       <c r="AL9" s="34">
         <f t="shared" si="22"/>
-        <v>99924</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="10" spans="1:39">
@@ -5560,7 +5555,7 @@
       </c>
       <c r="AH10" s="34">
         <f t="shared" si="20"/>
-        <v>99900</v>
+        <v>99980</v>
       </c>
       <c r="AI10" s="10" t="s">
         <v>172</v>
@@ -5570,11 +5565,11 @@
       </c>
       <c r="AK10" s="34">
         <f t="shared" si="21"/>
-        <v>99900</v>
+        <v>99980</v>
       </c>
       <c r="AL10" s="34">
         <f t="shared" si="22"/>
-        <v>99920</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="11" spans="1:39">
@@ -5690,7 +5685,7 @@
       </c>
       <c r="AH11" s="34">
         <f t="shared" si="20"/>
-        <v>99895</v>
+        <v>99979</v>
       </c>
       <c r="AI11" s="10" t="s">
         <v>172</v>
@@ -5700,11 +5695,11 @@
       </c>
       <c r="AK11" s="34">
         <f t="shared" si="21"/>
-        <v>99895</v>
+        <v>99979</v>
       </c>
       <c r="AL11" s="34">
         <f t="shared" si="22"/>
-        <v>99916</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="12" spans="1:39">
@@ -5820,7 +5815,7 @@
       </c>
       <c r="AH12" s="102">
         <f t="shared" si="20"/>
-        <v>99890</v>
+        <v>99978</v>
       </c>
       <c r="AI12" s="10" t="s">
         <v>172</v>
@@ -5830,11 +5825,11 @@
       </c>
       <c r="AK12" s="102">
         <f t="shared" si="21"/>
-        <v>99890</v>
+        <v>99978</v>
       </c>
       <c r="AL12" s="102">
         <f t="shared" si="22"/>
-        <v>99912</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="13" spans="1:39">
@@ -5950,7 +5945,7 @@
       </c>
       <c r="AH13" s="34">
         <f t="shared" si="20"/>
-        <v>99885</v>
+        <v>99977</v>
       </c>
       <c r="AI13" s="10" t="s">
         <v>172</v>
@@ -5960,11 +5955,11 @@
       </c>
       <c r="AK13" s="34">
         <f t="shared" si="21"/>
-        <v>99885</v>
+        <v>99977</v>
       </c>
       <c r="AL13" s="34">
         <f t="shared" si="22"/>
-        <v>99908</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="14" spans="1:39">
@@ -6080,7 +6075,7 @@
       </c>
       <c r="AH14" s="34">
         <f t="shared" si="20"/>
-        <v>99880</v>
+        <v>99976</v>
       </c>
       <c r="AI14" s="10" t="s">
         <v>172</v>
@@ -6090,11 +6085,11 @@
       </c>
       <c r="AK14" s="34">
         <f t="shared" si="21"/>
-        <v>99880</v>
+        <v>99976</v>
       </c>
       <c r="AL14" s="34">
         <f t="shared" si="22"/>
-        <v>99904</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="15" spans="1:39" s="23" customFormat="1">
@@ -7253,11 +7248,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
-        <v>90841</v>
+        <v>99656</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -7267,11 +7262,11 @@
       </c>
       <c r="AK5" s="33">
         <f>AH5</f>
-        <v>90841</v>
+        <v>99656</v>
       </c>
       <c r="AL5" s="33">
         <f>AK5+G5</f>
-        <v>90856</v>
+        <v>99671</v>
       </c>
       <c r="AM5" s="28" t="s">
         <v>66</v>
@@ -7280,15 +7275,15 @@
         <v>175</v>
       </c>
       <c r="AO5" s="29" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
-        <v>99845</v>
+        <v>100001600</v>
       </c>
       <c r="AQ5" s="28">
         <f>AO5+AF5</f>
-        <v>99845</v>
+        <v>100001600</v>
       </c>
     </row>
     <row r="6" spans="1:43" ht="14.25" customHeight="1">
@@ -8185,7 +8180,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99861</v>
+        <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -8635,7 +8630,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99816</v>
+        <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -9085,7 +9080,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99806</v>
+        <v>80704</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -9543,7 +9538,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99891</v>
+        <v>82574</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -9676,7 +9671,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99965</v>
+        <v>9657.5</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -10132,7 +10127,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>-10</v>
+        <v>80704</v>
       </c>
       <c r="AI5" s="63" t="s">
         <v>175</v>
@@ -10579,7 +10574,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>-10</v>
+        <v>80704</v>
       </c>
       <c r="AI5" s="63" t="s">
         <v>75</v>
@@ -11029,11 +11024,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>95771</v>
+        <v>80699</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -11486,7 +11481,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99831</v>
+        <v>63733</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -11937,7 +11932,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99957.5</v>
+        <v>9630</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -12063,7 +12058,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99791</v>
+        <v>78219</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -12376,13 +12371,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -12496,7 +12491,7 @@
         <v>199</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>243</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -12504,13 +12499,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>82</v>
+        <v>209</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>82</v>
+        <v>209</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -12624,7 +12619,7 @@
         <v>199</v>
       </c>
       <c r="AL6" s="66" t="s">
-        <v>243</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -12927,13 +12922,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -13047,7 +13042,7 @@
         <v>199</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -13175,7 +13170,7 @@
         <v>199</v>
       </c>
       <c r="AL6" s="66" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -13583,7 +13578,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>-7.5</v>
+        <v>9612.5</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -14760,14 +14755,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -14775,7 +14770,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -14783,7 +14778,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -14799,7 +14794,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -14817,22 +14812,22 @@
       </c>
       <c r="Z5" s="9">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1176</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -14842,11 +14837,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99760</v>
+        <v>9645</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -14889,14 +14884,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -14904,7 +14899,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -14912,7 +14907,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -14928,7 +14923,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -14946,22 +14941,22 @@
       </c>
       <c r="Z6" s="9">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>896</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -14971,11 +14966,11 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99920</v>
+        <v>9950.6589999999997</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -15432,25 +15427,25 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>99695</v>
+        <v>49586</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>173</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>99695</v>
+        <v>49586</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>99710</v>
+        <v>49601</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -15895,25 +15890,25 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
-        <v>99710</v>
+        <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>173</v>
       </c>
       <c r="AK5" s="34">
         <f>AH5</f>
-        <v>99710</v>
+        <v>65983</v>
       </c>
       <c r="AL5" s="34">
         <f>AK5+G5</f>
-        <v>99725</v>
+        <v>65998</v>
       </c>
       <c r="AM5" s="59"/>
     </row>
@@ -16012,7 +16007,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>128</v>
@@ -16082,7 +16077,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>127</v>
@@ -16238,7 +16233,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16393,7 +16388,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16546,7 +16541,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16854,7 +16849,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="166" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -17009,7 +17004,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -17340,14 +17335,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -17355,7 +17350,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -17363,7 +17358,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -17379,7 +17374,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -17405,14 +17400,14 @@
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -17426,7 +17421,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99970</v>
+        <v>9745</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -17469,14 +17464,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -17484,7 +17479,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -17492,7 +17487,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -17508,7 +17503,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -17534,14 +17529,14 @@
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -17555,7 +17550,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99990</v>
+        <v>9880</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -17752,7 +17747,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17907,7 +17902,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -18767,22 +18762,22 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>32</v>
@@ -18795,11 +18790,11 @@
       </c>
       <c r="O5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
-        <v>20.25</v>
+        <v>40.5</v>
       </c>
       <c r="P5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
-        <v>20.25</v>
+        <v>40.5</v>
       </c>
       <c r="Q5" s="34">
         <f>IF($D$3=2,ROUND((K5*N5),2),0)</f>
@@ -18811,11 +18806,11 @@
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>40.5</v>
+        <v>81</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -19109,7 +19104,7 @@
         <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>57</v>
+        <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -19121,22 +19116,22 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>219</v>
+        <v>242</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>32</v>
@@ -19157,7 +19152,7 @@
       </c>
       <c r="Q5" s="34">
         <f>IF($D$3=2,ROUND((K5*N5),2),0)</f>
-        <v>40.5</v>
+        <v>81</v>
       </c>
       <c r="R5" s="34">
         <f>IF($D$3=4,ROUND((K5*N5),2),0)</f>
@@ -19165,11 +19160,11 @@
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>40.5</v>
+        <v>81</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>265.5</v>
+        <v>531</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -19462,8 +19457,8 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>163</v>
+      <c r="C5" s="29">
+        <v>20</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -19475,7 +19470,7 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>54</v>
+        <v>242</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
@@ -19486,11 +19481,11 @@
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>32</v>
@@ -19503,7 +19498,7 @@
       </c>
       <c r="O5" s="34">
         <f>IF(OR($D$3=1,$D$3=4),ROUND(((K5*N5)/2),2),0)</f>
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="P5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
@@ -19515,15 +19510,15 @@
       </c>
       <c r="R5" s="34">
         <f>IF($D$3=4,ROUND(((K5*N5)/2),2),0)</f>
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>708</v>
+        <v>472</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -19829,7 +19824,7 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
@@ -19840,11 +19835,11 @@
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>17.5</v>
+        <v>30</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>437.5</v>
+        <v>750</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>32</v>
@@ -19857,7 +19852,7 @@
       </c>
       <c r="O5" s="34">
         <f>IF(OR($D$3=1,$D$3=4),ROUND(((K5*N5)/2),2),0)</f>
-        <v>39.380000000000003</v>
+        <v>67.5</v>
       </c>
       <c r="P5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
@@ -19869,15 +19864,15 @@
       </c>
       <c r="R5" s="34">
         <f>IF($D$3=4,ROUND(((K5*N5)/2),2),0)</f>
-        <v>39.380000000000003</v>
+        <v>67.5</v>
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>78.760000000000005</v>
+        <v>135</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>437.5</v>
+        <v>750</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -20242,14 +20237,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -20257,7 +20252,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -20265,7 +20260,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -20281,7 +20276,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -20299,22 +20294,22 @@
       </c>
       <c r="Z5" s="9">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1008</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -20328,7 +20323,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99940</v>
+        <v>9717</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -20371,14 +20366,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -20386,7 +20381,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -20394,7 +20389,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -20410,7 +20405,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -20428,22 +20423,22 @@
       </c>
       <c r="Z6" s="9">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>784</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -20457,7 +20452,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99980</v>
+        <v>9865</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -20759,7 +20754,7 @@
         <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>139</v>
+        <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -20771,25 +20766,25 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>160</v>
+        <v>127</v>
       </c>
       <c r="I5" s="10">
         <f>ROUND(C5*H5/F5,3)</f>
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>17.5</v>
+        <v>22.5</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>437.5</v>
+        <v>450</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>32</v>
+        <v>159</v>
       </c>
       <c r="M5" s="33">
         <v>88363221</v>
@@ -20807,7 +20802,7 @@
       </c>
       <c r="Q5" s="34">
         <f>IF($D$3=2,ROUND((K5*N5),2),0)</f>
-        <v>78.75</v>
+        <v>81</v>
       </c>
       <c r="R5" s="34">
         <f>IF($D$3=4,ROUND((K5*N5),2),0)</f>
@@ -20815,11 +20810,11 @@
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>78.75</v>
+        <v>81</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>437.5</v>
+        <v>450</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -21125,7 +21120,7 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
@@ -21136,11 +21131,11 @@
       </c>
       <c r="J5" s="10">
         <f>I5*(G5/C5)</f>
-        <v>17.5</v>
+        <v>20</v>
       </c>
       <c r="K5" s="10">
         <f>I5*G5</f>
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="L5" s="29" t="s">
         <v>32</v>
@@ -21153,11 +21148,11 @@
       </c>
       <c r="O5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
-        <v>31.5</v>
+        <v>36</v>
       </c>
       <c r="P5" s="34">
         <f>IF($D$3=1,ROUND(((K5*N5)/2),2),0)</f>
-        <v>31.5</v>
+        <v>36</v>
       </c>
       <c r="Q5" s="34">
         <f>IF($D$3=2,ROUND((K5*N5),2),0)</f>
@@ -21169,11 +21164,11 @@
       </c>
       <c r="S5" s="34">
         <f>ROUND(O5+P5+Q5+R5,2)</f>
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="T5" s="34">
         <f>ROUND(IF($J$3=1, K5+S5, K5),2)</f>
-        <v>413</v>
+        <v>472</v>
       </c>
       <c r="U5" s="59"/>
       <c r="AH5" s="29"/>
@@ -21254,13 +21249,13 @@
       <c r="D1" s="173"/>
     </row>
     <row r="2" spans="1:17" ht="18">
-      <c r="D2" s="109"/>
+      <c r="D2" s="171"/>
     </row>
     <row r="3" spans="1:17" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="108"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
     </row>
     <row r="4" spans="1:17" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
@@ -21320,7 +21315,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>122</v>
+        <v>243</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>139</v>
@@ -21386,6 +21381,165 @@
 </file>
 
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="13" style="29" customWidth="1"/>
+    <col min="11" max="14" width="9.140625" style="29"/>
+    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="29"/>
+    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="27.75" customHeight="1">
+      <c r="A1" s="173" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+    </row>
+    <row r="2" spans="1:17" ht="18">
+      <c r="D2" s="109"/>
+    </row>
+    <row r="3" spans="1:17" ht="19.899999999999999" customHeight="1">
+      <c r="A3" s="172"/>
+      <c r="B3" s="172"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="108"/>
+    </row>
+    <row r="4" spans="1:17" s="31" customFormat="1">
+      <c r="A4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="113" t="s">
+        <v>133</v>
+      </c>
+      <c r="F4" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="115" t="s">
+        <v>126</v>
+      </c>
+      <c r="H4" s="115" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="115" t="s">
+        <v>149</v>
+      </c>
+      <c r="J4" s="115" t="s">
+        <v>150</v>
+      </c>
+      <c r="K4" s="115" t="s">
+        <v>151</v>
+      </c>
+      <c r="L4" s="115" t="s">
+        <v>152</v>
+      </c>
+      <c r="M4" s="115" t="s">
+        <v>153</v>
+      </c>
+      <c r="N4" s="115" t="s">
+        <v>158</v>
+      </c>
+      <c r="O4" s="115" t="s">
+        <v>89</v>
+      </c>
+      <c r="P4" s="115" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q4" s="115" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="15">
+      <c r="A5" s="10">
+        <v>1</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>134</v>
+      </c>
+      <c r="F5" s="10">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10">
+        <v>20</v>
+      </c>
+      <c r="H5" s="10">
+        <v>1</v>
+      </c>
+      <c r="I5" s="10">
+        <f>ROUND(C5*H5/F5,3)</f>
+        <v>25</v>
+      </c>
+      <c r="J5" s="122">
+        <f>I5*(G5/C5)</f>
+        <v>20</v>
+      </c>
+      <c r="K5" s="10">
+        <f>I5*G5</f>
+        <v>500</v>
+      </c>
+      <c r="L5" s="124">
+        <v>0.18</v>
+      </c>
+      <c r="M5" s="10">
+        <f>K5*L5</f>
+        <v>90</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="O5" s="123">
+        <v>88363221</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q5" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="L6" s="28"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
@@ -21401,7 +21555,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
       <c r="A1" s="173" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B1" s="173"/>
       <c r="C1" s="173"/>
@@ -21412,51 +21566,51 @@
     </row>
     <row r="3" spans="1:8" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="174" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B3" s="174"/>
       <c r="C3" s="174"/>
       <c r="D3" s="174"/>
       <c r="E3" s="175" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F3" s="175"/>
     </row>
     <row r="4" spans="1:8" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>228</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15">
       <c r="A5" s="122" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D5" s="10">
         <v>11</v>
       </c>
       <c r="E5" s="122" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F5" s="114" t="s">
         <v>160</v>
@@ -21476,7 +21630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
@@ -21830,7 +21984,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AL8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
@@ -21909,7 +22063,7 @@
     </row>
     <row r="2" spans="1:38" ht="18">
       <c r="A2" s="134" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B2" s="134"/>
       <c r="C2" s="134"/>
@@ -21953,7 +22107,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="140" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F3" s="141"/>
       <c r="G3" s="141"/>
@@ -22182,7 +22336,7 @@
         <v>11493.38</v>
       </c>
       <c r="V5" s="155" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W5" s="156">
         <v>0.18</v>
@@ -22247,13 +22401,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C6" s="155">
         <v>0</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E6" s="155" t="s">
         <v>159</v>
@@ -22317,7 +22471,7 @@
         <v>26656.080000000002</v>
       </c>
       <c r="V6" s="155" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W6" s="156">
         <v>0.18</v>
@@ -22395,7 +22549,7 @@
       <c r="O7" s="159"/>
       <c r="P7" s="161"/>
       <c r="Q7" s="161" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="R7" s="161"/>
       <c r="S7" s="161"/>
@@ -22406,7 +22560,7 @@
       <c r="X7" s="159"/>
       <c r="Y7" s="159"/>
       <c r="Z7" s="161" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AA7" s="161"/>
       <c r="AB7" s="162">
@@ -22414,7 +22568,7 @@
         <v>45016.36</v>
       </c>
       <c r="AC7" s="161" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AD7" s="162">
         <f>SUM(AD5:AD6)</f>
@@ -22464,1416 +22618,6 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A3:B3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AL6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="173" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="173"/>
-      <c r="C1" s="173"/>
-      <c r="D1" s="173"/>
-      <c r="E1" s="173"/>
-      <c r="F1" s="173"/>
-      <c r="G1" s="173"/>
-      <c r="H1" s="173"/>
-      <c r="I1" s="173"/>
-      <c r="J1" s="173"/>
-      <c r="K1" s="173"/>
-      <c r="L1" s="173"/>
-      <c r="M1" s="173"/>
-      <c r="N1" s="173"/>
-      <c r="O1" s="173"/>
-      <c r="P1" s="173"/>
-      <c r="Q1" s="173"/>
-      <c r="R1" s="173"/>
-      <c r="S1" s="173"/>
-      <c r="T1" s="173"/>
-      <c r="U1" s="173"/>
-      <c r="V1" s="173"/>
-      <c r="W1" s="173"/>
-      <c r="X1" s="173"/>
-      <c r="Y1" s="173"/>
-      <c r="Z1" s="173"/>
-      <c r="AA1" s="173"/>
-      <c r="AB1" s="173"/>
-      <c r="AC1" s="171"/>
-      <c r="AD1" s="171"/>
-      <c r="AE1" s="171"/>
-      <c r="AF1" s="171"/>
-      <c r="AG1" s="27"/>
-    </row>
-    <row r="2" spans="1:38" ht="18">
-      <c r="A2" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
-      <c r="O2" s="171"/>
-      <c r="P2" s="171"/>
-      <c r="Q2" s="171"/>
-      <c r="R2" s="171"/>
-      <c r="S2" s="171"/>
-      <c r="T2" s="171"/>
-      <c r="U2" s="171"/>
-      <c r="V2" s="171"/>
-      <c r="W2" s="171"/>
-      <c r="X2" s="171"/>
-      <c r="Y2" s="171"/>
-      <c r="Z2" s="171"/>
-      <c r="AA2" s="171"/>
-      <c r="AB2" s="171"/>
-      <c r="AC2" s="171"/>
-      <c r="AD2" s="171"/>
-      <c r="AE2" s="171"/>
-      <c r="AF2" s="171"/>
-      <c r="AG2" s="27"/>
-    </row>
-    <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="172" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="172"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="3">
-        <v>1</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="7">
-        <v>1</v>
-      </c>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="6"/>
-      <c r="AG3" s="30"/>
-    </row>
-    <row r="4" spans="1:38" s="31" customFormat="1" ht="28.5">
-      <c r="A4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="O4" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P4" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q4" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="T4" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="W4" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="X4" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA4" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC4" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AE4" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF4" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH4" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI4" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ4" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="AK4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL4" s="20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:38" ht="15">
-      <c r="A5" s="10">
-        <v>1</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="10">
-        <v>0</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="33">
-        <v>15</v>
-      </c>
-      <c r="H5" s="9">
-        <v>1500</v>
-      </c>
-      <c r="I5" s="9">
-        <f>G5*H5</f>
-        <v>22500</v>
-      </c>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="9">
-        <f>I5</f>
-        <v>22500</v>
-      </c>
-      <c r="N5" s="9">
-        <f>ROUND((M5*J5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="9">
-        <f>I5-N5</f>
-        <v>22500</v>
-      </c>
-      <c r="P5" s="9">
-        <f>ROUND((O5*K5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="9">
-        <f>ROUND(O5-P5,2)</f>
-        <v>22500</v>
-      </c>
-      <c r="R5" s="9">
-        <f>ROUND((Q5*L5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="S5" s="35">
-        <f>N5+P5+R5</f>
-        <v>0</v>
-      </c>
-      <c r="T5" s="35">
-        <f>S5/G5</f>
-        <v>0</v>
-      </c>
-      <c r="U5" s="9">
-        <f>(I5-S5)</f>
-        <v>22500</v>
-      </c>
-      <c r="V5" s="33">
-        <v>88363222</v>
-      </c>
-      <c r="W5" s="22">
-        <v>0.18</v>
-      </c>
-      <c r="X5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>2025</v>
-      </c>
-      <c r="Y5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>2025</v>
-      </c>
-      <c r="Z5" s="9">
-        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="9">
-        <f>X5+Y5+Z5</f>
-        <v>4050</v>
-      </c>
-      <c r="AB5" s="9">
-        <f>U5+AA5</f>
-        <v>26550</v>
-      </c>
-      <c r="AC5" s="9">
-        <v>120</v>
-      </c>
-      <c r="AD5" s="9">
-        <f t="shared" ref="AD5" si="0">U5*$N$3</f>
-        <v>22500</v>
-      </c>
-      <c r="AE5" s="8">
-        <v>1</v>
-      </c>
-      <c r="AF5" s="9">
-        <f t="shared" ref="AF5" si="1">G5/AE5</f>
-        <v>15</v>
-      </c>
-      <c r="AG5" s="36" t="s">
-        <v>244</v>
-      </c>
-      <c r="AH5" s="9">
-        <f>AG5-AF5</f>
-        <v>90991</v>
-      </c>
-      <c r="AI5" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="AK5" s="29">
-        <v>87850</v>
-      </c>
-      <c r="AL5" s="33">
-        <f>AK5+G5</f>
-        <v>87865</v>
-      </c>
-    </row>
-    <row r="6" spans="1:38" ht="14.25" customHeight="1">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="94">
-        <f>SUM(I5:I5)</f>
-        <v>22500</v>
-      </c>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="25"/>
-      <c r="U6" s="94">
-        <f>SUM(U5:U5)</f>
-        <v>22500</v>
-      </c>
-      <c r="V6" s="25"/>
-      <c r="W6" s="26"/>
-      <c r="X6" s="25"/>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="94">
-        <f>SUM(AA5:AA5)</f>
-        <v>4050</v>
-      </c>
-      <c r="AB6" s="94">
-        <f>SUM(AB5:AB5)</f>
-        <v>26550</v>
-      </c>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="25"/>
-      <c r="AE6" s="24"/>
-      <c r="AF6" s="25"/>
-      <c r="AG6" s="25"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:AB1"/>
-    <mergeCell ref="A3:B3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AL6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="173" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="173"/>
-      <c r="C1" s="173"/>
-      <c r="D1" s="173"/>
-      <c r="E1" s="173"/>
-      <c r="F1" s="173"/>
-      <c r="G1" s="173"/>
-      <c r="H1" s="173"/>
-      <c r="I1" s="173"/>
-      <c r="J1" s="173"/>
-      <c r="K1" s="173"/>
-      <c r="L1" s="173"/>
-      <c r="M1" s="173"/>
-      <c r="N1" s="173"/>
-      <c r="O1" s="173"/>
-      <c r="P1" s="173"/>
-      <c r="Q1" s="173"/>
-      <c r="R1" s="173"/>
-      <c r="S1" s="173"/>
-      <c r="T1" s="173"/>
-      <c r="U1" s="173"/>
-      <c r="V1" s="173"/>
-      <c r="W1" s="173"/>
-      <c r="X1" s="173"/>
-      <c r="Y1" s="173"/>
-      <c r="Z1" s="173"/>
-      <c r="AA1" s="173"/>
-      <c r="AB1" s="173"/>
-      <c r="AC1" s="171"/>
-      <c r="AD1" s="171"/>
-      <c r="AE1" s="171"/>
-      <c r="AF1" s="171"/>
-      <c r="AG1" s="27"/>
-    </row>
-    <row r="2" spans="1:38" ht="18">
-      <c r="A2" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
-      <c r="O2" s="171"/>
-      <c r="P2" s="171"/>
-      <c r="Q2" s="171"/>
-      <c r="R2" s="171"/>
-      <c r="S2" s="171"/>
-      <c r="T2" s="171"/>
-      <c r="U2" s="171"/>
-      <c r="V2" s="171"/>
-      <c r="W2" s="171"/>
-      <c r="X2" s="171"/>
-      <c r="Y2" s="171"/>
-      <c r="Z2" s="171"/>
-      <c r="AA2" s="171"/>
-      <c r="AB2" s="171"/>
-      <c r="AC2" s="171"/>
-      <c r="AD2" s="171"/>
-      <c r="AE2" s="171"/>
-      <c r="AF2" s="171"/>
-      <c r="AG2" s="27"/>
-    </row>
-    <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="172" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="172"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="3">
-        <v>3</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="7">
-        <v>1</v>
-      </c>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="6"/>
-      <c r="AG3" s="30"/>
-    </row>
-    <row r="4" spans="1:38" s="31" customFormat="1" ht="28.5">
-      <c r="A4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="O4" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P4" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q4" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="T4" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="W4" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="X4" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA4" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC4" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AE4" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF4" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH4" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI4" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ4" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="AK4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL4" s="20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:38" ht="15">
-      <c r="A5" s="10">
-        <v>1</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="10">
-        <v>0</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="33">
-        <v>15</v>
-      </c>
-      <c r="H5" s="9">
-        <v>110</v>
-      </c>
-      <c r="I5" s="9">
-        <f>G5*H5</f>
-        <v>1650</v>
-      </c>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="9">
-        <f>I5</f>
-        <v>1650</v>
-      </c>
-      <c r="N5" s="9">
-        <f>ROUND((M5*J5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="9">
-        <f>I5-N5</f>
-        <v>1650</v>
-      </c>
-      <c r="P5" s="9">
-        <f>ROUND((O5*K5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="9">
-        <f>ROUND(O5-P5,2)</f>
-        <v>1650</v>
-      </c>
-      <c r="R5" s="9">
-        <f>ROUND((Q5*L5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="S5" s="35">
-        <f>N5+P5+R5</f>
-        <v>0</v>
-      </c>
-      <c r="T5" s="35">
-        <f>S5/G5</f>
-        <v>0</v>
-      </c>
-      <c r="U5" s="9">
-        <f>(I5-S5)</f>
-        <v>1650</v>
-      </c>
-      <c r="V5" s="33">
-        <v>88363222</v>
-      </c>
-      <c r="W5" s="22">
-        <v>0.18</v>
-      </c>
-      <c r="X5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="9">
-        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="9">
-        <f>X5+Y5+Z5</f>
-        <v>0</v>
-      </c>
-      <c r="AB5" s="9">
-        <f>U5+AA5</f>
-        <v>1650</v>
-      </c>
-      <c r="AC5" s="9">
-        <v>120</v>
-      </c>
-      <c r="AD5" s="9">
-        <f t="shared" ref="AD5" si="0">U5*$N$3</f>
-        <v>1650</v>
-      </c>
-      <c r="AE5" s="8">
-        <v>1</v>
-      </c>
-      <c r="AF5" s="9">
-        <f t="shared" ref="AF5" si="1">G5/AE5</f>
-        <v>15</v>
-      </c>
-      <c r="AG5" s="36" t="s">
-        <v>245</v>
-      </c>
-      <c r="AH5" s="9">
-        <f>AG5-AF5</f>
-        <v>93801</v>
-      </c>
-      <c r="AI5" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="AK5" s="29">
-        <v>87850</v>
-      </c>
-      <c r="AL5" s="33">
-        <f>AK5+G5</f>
-        <v>87865</v>
-      </c>
-    </row>
-    <row r="6" spans="1:38" ht="14.25" customHeight="1">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="94">
-        <f>SUM(I5:I5)</f>
-        <v>1650</v>
-      </c>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="25"/>
-      <c r="U6" s="94">
-        <f>SUM(U5:U5)</f>
-        <v>1650</v>
-      </c>
-      <c r="V6" s="25"/>
-      <c r="W6" s="26"/>
-      <c r="X6" s="25"/>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="94">
-        <f>SUM(AA5:AA5)</f>
-        <v>0</v>
-      </c>
-      <c r="AB6" s="94">
-        <f>SUM(AB5:AB5)</f>
-        <v>1650</v>
-      </c>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="25"/>
-      <c r="AE6" s="24"/>
-      <c r="AF6" s="25"/>
-      <c r="AG6" s="25"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:AB1"/>
-    <mergeCell ref="A3:B3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AL6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="173" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="173"/>
-      <c r="C1" s="173"/>
-      <c r="D1" s="173"/>
-      <c r="E1" s="173"/>
-      <c r="F1" s="173"/>
-      <c r="G1" s="173"/>
-      <c r="H1" s="173"/>
-      <c r="I1" s="173"/>
-      <c r="J1" s="173"/>
-      <c r="K1" s="173"/>
-      <c r="L1" s="173"/>
-      <c r="M1" s="173"/>
-      <c r="N1" s="173"/>
-      <c r="O1" s="173"/>
-      <c r="P1" s="173"/>
-      <c r="Q1" s="173"/>
-      <c r="R1" s="173"/>
-      <c r="S1" s="173"/>
-      <c r="T1" s="173"/>
-      <c r="U1" s="173"/>
-      <c r="V1" s="173"/>
-      <c r="W1" s="173"/>
-      <c r="X1" s="173"/>
-      <c r="Y1" s="173"/>
-      <c r="Z1" s="173"/>
-      <c r="AA1" s="173"/>
-      <c r="AB1" s="173"/>
-      <c r="AC1" s="171"/>
-      <c r="AD1" s="171"/>
-      <c r="AE1" s="171"/>
-      <c r="AF1" s="171"/>
-      <c r="AG1" s="27"/>
-    </row>
-    <row r="2" spans="1:38" ht="18">
-      <c r="A2" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
-      <c r="O2" s="171"/>
-      <c r="P2" s="171"/>
-      <c r="Q2" s="171"/>
-      <c r="R2" s="171"/>
-      <c r="S2" s="171"/>
-      <c r="T2" s="171"/>
-      <c r="U2" s="171"/>
-      <c r="V2" s="171"/>
-      <c r="W2" s="171"/>
-      <c r="X2" s="171"/>
-      <c r="Y2" s="171"/>
-      <c r="Z2" s="171"/>
-      <c r="AA2" s="171"/>
-      <c r="AB2" s="171"/>
-      <c r="AC2" s="171"/>
-      <c r="AD2" s="171"/>
-      <c r="AE2" s="171"/>
-      <c r="AF2" s="171"/>
-      <c r="AG2" s="27"/>
-    </row>
-    <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="172" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="172"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="3">
-        <v>2</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="7">
-        <v>1</v>
-      </c>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="6"/>
-      <c r="AG3" s="30"/>
-    </row>
-    <row r="4" spans="1:38" s="31" customFormat="1" ht="28.5">
-      <c r="A4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="O4" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P4" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q4" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="T4" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="W4" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="X4" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA4" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC4" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AE4" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF4" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH4" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI4" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ4" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="AK4" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL4" s="20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:38" ht="15">
-      <c r="A5" s="10">
-        <v>1</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="10">
-        <v>0</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="33">
-        <v>15</v>
-      </c>
-      <c r="H5" s="9">
-        <v>1500</v>
-      </c>
-      <c r="I5" s="9">
-        <f>G5*H5</f>
-        <v>22500</v>
-      </c>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="9">
-        <f>I5</f>
-        <v>22500</v>
-      </c>
-      <c r="N5" s="9">
-        <f>ROUND((M5*J5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="9">
-        <f>I5-N5</f>
-        <v>22500</v>
-      </c>
-      <c r="P5" s="9">
-        <f>ROUND((O5*K5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="9">
-        <f>ROUND(O5-P5,2)</f>
-        <v>22500</v>
-      </c>
-      <c r="R5" s="9">
-        <f>ROUND((Q5*L5)/100,2)</f>
-        <v>0</v>
-      </c>
-      <c r="S5" s="35">
-        <f>N5+P5+R5</f>
-        <v>0</v>
-      </c>
-      <c r="T5" s="35">
-        <f>S5/G5</f>
-        <v>0</v>
-      </c>
-      <c r="U5" s="9">
-        <f>(I5-S5)</f>
-        <v>22500</v>
-      </c>
-      <c r="V5" s="33">
-        <v>88363222</v>
-      </c>
-      <c r="W5" s="22">
-        <v>0.18</v>
-      </c>
-      <c r="X5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="9">
-        <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="9">
-        <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>4050</v>
-      </c>
-      <c r="AA5" s="9">
-        <f>X5+Y5+Z5</f>
-        <v>4050</v>
-      </c>
-      <c r="AB5" s="9">
-        <f>U5+AA5</f>
-        <v>26550</v>
-      </c>
-      <c r="AC5" s="9">
-        <v>120</v>
-      </c>
-      <c r="AD5" s="9">
-        <f t="shared" ref="AD5" si="0">U5*$N$3</f>
-        <v>22500</v>
-      </c>
-      <c r="AE5" s="8">
-        <v>1</v>
-      </c>
-      <c r="AF5" s="9">
-        <f t="shared" ref="AF5" si="1">G5/AE5</f>
-        <v>15</v>
-      </c>
-      <c r="AG5" s="36" t="s">
-        <v>246</v>
-      </c>
-      <c r="AH5" s="9">
-        <f>AG5-AF5</f>
-        <v>91006</v>
-      </c>
-      <c r="AI5" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="AJ5" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="AK5" s="29">
-        <v>87850</v>
-      </c>
-      <c r="AL5" s="33">
-        <f>AK5+G5</f>
-        <v>87865</v>
-      </c>
-    </row>
-    <row r="6" spans="1:38" ht="14.25" customHeight="1">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="94">
-        <f>SUM(I5:I5)</f>
-        <v>22500</v>
-      </c>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="25"/>
-      <c r="U6" s="94">
-        <f>SUM(U5:U5)</f>
-        <v>22500</v>
-      </c>
-      <c r="V6" s="25"/>
-      <c r="W6" s="26"/>
-      <c r="X6" s="25"/>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="94">
-        <f>SUM(AA5:AA5)</f>
-        <v>4050</v>
-      </c>
-      <c r="AB6" s="94">
-        <f>SUM(AB5:AB5)</f>
-        <v>26550</v>
-      </c>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="25"/>
-      <c r="AE6" s="24"/>
-      <c r="AF6" s="25"/>
-      <c r="AG6" s="25"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:AB1"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24192,14 +22936,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -24207,7 +22951,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -24215,7 +22959,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -24231,7 +22975,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -24257,14 +23001,14 @@
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -24278,7 +23022,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99940</v>
+        <v>9795</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -24321,14 +23065,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -24336,7 +23080,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -24344,7 +23088,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -24360,7 +23104,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -24386,14 +23130,14 @@
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -24407,7 +23151,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99983.334000000003</v>
+        <v>9900</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -24780,14 +23524,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -24795,7 +23539,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -24803,7 +23547,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -24819,7 +23563,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -24837,22 +23581,22 @@
       </c>
       <c r="Z5" s="9">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>109.8</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>109.8</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1024.8</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>915</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -24866,7 +23610,7 @@
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99940</v>
+        <v>9703</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -24909,14 +23653,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -24924,7 +23668,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -24932,7 +23676,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -24948,7 +23692,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -24966,22 +23710,22 @@
       </c>
       <c r="Z6" s="9">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>85.2</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>85.2</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>795.2</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -24995,7 +23739,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99980</v>
+        <v>9852.5</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -25364,18 +24108,18 @@
         <v>15</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -25383,7 +24127,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -25391,7 +24135,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -25407,7 +24151,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -25433,14 +24177,14 @@
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>1215</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -25450,11 +24194,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99850</v>
+        <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -25497,14 +24241,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -25512,7 +24256,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -25520,7 +24264,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -25536,7 +24280,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -25562,14 +24306,14 @@
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -25583,7 +24327,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99950</v>
+        <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>
@@ -25956,14 +24700,14 @@
       </c>
       <c r="I5" s="9">
         <f>G5*H5</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="J5" s="34"/>
       <c r="K5" s="34"/>
       <c r="L5" s="34"/>
       <c r="M5" s="9">
         <f>I5</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="N5" s="9">
         <f>ROUND((M5*J5)/100,2)</f>
@@ -25971,7 +24715,7 @@
       </c>
       <c r="O5" s="9">
         <f>I5-N5</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="P5" s="9">
         <f>ROUND((O5*K5)/100,2)</f>
@@ -25979,7 +24723,7 @@
       </c>
       <c r="Q5" s="9">
         <f>ROUND(O5-P5,2)</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="R5" s="9">
         <f>ROUND((Q5*L5)/100,2)</f>
@@ -25995,7 +24739,7 @@
       </c>
       <c r="U5" s="9">
         <f>(I5-S5)</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="V5" s="33">
         <v>88363222</v>
@@ -26013,22 +24757,22 @@
       </c>
       <c r="Z5" s="9">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="9">
         <f>X5+Y5+Z5</f>
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="9">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="9">
         <v>120</v>
       </c>
       <c r="AD5" s="9">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="8">
         <v>1</v>
@@ -26038,11 +24782,11 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
-        <v>99879</v>
+        <v>9805</v>
       </c>
       <c r="AI5" s="10" t="s">
         <v>172</v>
@@ -26085,14 +24829,14 @@
       </c>
       <c r="I6" s="9">
         <f>G6*H6</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
       <c r="L6" s="34"/>
       <c r="M6" s="9">
         <f>I6</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="N6" s="9">
         <f>ROUND((M6*J6)/100,2)</f>
@@ -26100,7 +24844,7 @@
       </c>
       <c r="O6" s="9">
         <f>I6-N6</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="P6" s="9">
         <f>ROUND((O6*K6)/100,2)</f>
@@ -26108,7 +24852,7 @@
       </c>
       <c r="Q6" s="9">
         <f>ROUND(O6-P6,2)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="R6" s="9">
         <f>ROUND((Q6*L6)/100,2)</f>
@@ -26124,7 +24868,7 @@
       </c>
       <c r="U6" s="9">
         <f>(I6-S6)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="V6" s="33">
         <v>88363222</v>
@@ -26142,22 +24886,22 @@
       </c>
       <c r="Z6" s="9">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="9">
         <f>X6+Y6+Z6</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="9">
         <f t="shared" si="0"/>
-        <v>560</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="9">
         <v>120</v>
       </c>
       <c r="AD6" s="9">
         <f t="shared" si="1"/>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="8">
         <v>2</v>
@@ -26171,7 +24915,7 @@
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
-        <v>99960</v>
+        <v>9905</v>
       </c>
       <c r="AI6" s="10" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Subcontract Function With DB Validation Changes fixes
Subcontract Function With DB Validation Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="49" activeTab="51"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="47" activeTab="49"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2693" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="250">
   <si>
     <t>GST Sales</t>
   </si>
@@ -1822,43 +1822,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="14.0"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2410,43 +2410,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2984,44 +2984,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3447,44 +3447,44 @@
   <dimension ref="A1:AM13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="18.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4075,44 +4075,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4538,44 +4538,44 @@
   <dimension ref="A1:AM36"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -6868,48 +6868,48 @@
   <dimension ref="A1:AQ6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="36" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="41" width="14.140625" style="29" customWidth="1"/>
-    <col min="42" max="42" width="15" style="29" customWidth="1"/>
-    <col min="43" max="43" width="16.5703125" style="29" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="36.0"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="41" customWidth="true" style="29" width="14.140625"/>
+    <col min="42" max="42" customWidth="true" style="29" width="15.0"/>
+    <col min="43" max="43" customWidth="true" style="29" width="16.5703125"/>
+    <col min="44" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
@@ -7365,43 +7365,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.5703125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="21.28515625" style="29" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="34.5703125"/>
+    <col min="8" max="8" customWidth="true" style="29" width="21.28515625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -7820,43 +7820,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8270,43 +8270,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8720,43 +8720,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9170,44 +9170,44 @@
   <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -9770,43 +9770,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10217,43 +10217,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10664,43 +10664,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -11123,42 +11123,42 @@
   <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.42578125" style="29" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="15.42578125"/>
+    <col min="38" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
@@ -11570,43 +11570,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12115,43 +12115,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12666,43 +12666,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13217,43 +13217,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13637,43 +13637,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14057,43 +14057,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="11.7109375" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="11.7109375"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14477,43 +14477,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -15065,44 +15065,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15528,44 +15528,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15991,12 +15991,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16061,12 +16061,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16131,17 +16131,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16286,17 +16286,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16441,15 +16441,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="14.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="14.85546875"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16594,15 +16594,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16747,17 +16747,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16902,17 +16902,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17057,43 +17057,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -17645,17 +17645,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17800,17 +17800,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17955,12 +17955,12 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18093,17 +18093,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18248,17 +18248,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18403,14 +18403,14 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11" style="29" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.0"/>
+    <col min="11" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18543,45 +18543,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -18897,45 +18897,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19132,8 +19132,8 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>163</v>
+      <c r="C5" t="s" s="29">
+        <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -19141,13 +19141,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" t="s" s="29">
         <v>127</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="H5" s="29" t="s">
+      <c r="G5" t="s" s="29">
+        <v>167</v>
+      </c>
+      <c r="H5" t="s" s="29">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -19162,7 +19162,7 @@
         <f>I5*G5</f>
         <v>450</v>
       </c>
-      <c r="L5" s="29" t="s">
+      <c r="L5" t="s" s="29">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -19251,45 +19251,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19605,45 +19605,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19959,43 +19959,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -20547,45 +20547,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -20783,7 +20783,7 @@
         <v>122</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>139</v>
+        <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -20795,7 +20795,7 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>220</v>
+        <v>167</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
@@ -20901,45 +20901,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -21136,7 +21136,7 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" t="s" s="29">
         <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -21145,13 +21145,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" t="s" s="29">
         <v>127</v>
       </c>
-      <c r="G5" s="29" t="s">
+      <c r="G5" t="s" s="29">
         <v>220</v>
       </c>
-      <c r="H5" s="29" t="s">
+      <c r="H5" t="s" s="29">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -21166,7 +21166,7 @@
         <f>I5*G5</f>
         <v>400</v>
       </c>
-      <c r="L5" s="29" t="s">
+      <c r="L5" t="s" s="29">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -21255,18 +21255,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21350,7 +21350,7 @@
         <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="E5" s="67" t="s">
         <v>134</v>
@@ -21414,18 +21414,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21573,18 +21573,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21732,9 +21732,9 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
+    <col min="3" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1">
@@ -21758,10 +21758,10 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="29" t="s">
+      <c r="A5" t="s" s="29">
         <v>234</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" t="s" s="29">
         <v>232</v>
       </c>
     </row>
@@ -21783,13 +21783,13 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
+    <col min="3" max="3" customWidth="true" style="29" width="14.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="15.5703125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="7" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
@@ -21874,45 +21874,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -22228,40 +22228,40 @@
   <dimension ref="A1:AL8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="137" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="137" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="137" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="137" customWidth="1"/>
-    <col min="5" max="5" width="10" style="137" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="137" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="137" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="137" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="137" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="137" customWidth="1"/>
-    <col min="12" max="12" width="8" style="137" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="137" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="137" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="137" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="137" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="137" customWidth="1"/>
-    <col min="18" max="18" width="9" style="137" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="137" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="137" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="137" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" style="137" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="137" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="137" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="137" customWidth="1"/>
-    <col min="27" max="27" width="12" style="137" customWidth="1"/>
-    <col min="28" max="28" width="12.28515625" style="137" customWidth="1"/>
-    <col min="29" max="29" width="14.7109375" style="137" customWidth="1"/>
-    <col min="30" max="30" width="12.28515625" style="163" customWidth="1"/>
-    <col min="31" max="31" width="13.5703125" style="163" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.5703125" style="163" customWidth="1"/>
-    <col min="33" max="33" width="15.7109375" style="136" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.5703125" style="137" customWidth="1"/>
-    <col min="35" max="35" width="12.7109375" style="137" customWidth="1"/>
-    <col min="36" max="16384" width="9.140625" style="137"/>
+    <col min="1" max="1" customWidth="true" style="137" width="5.7109375"/>
+    <col min="2" max="2" customWidth="true" style="137" width="28.85546875"/>
+    <col min="3" max="3" customWidth="true" style="137" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="137" width="28.85546875"/>
+    <col min="5" max="5" customWidth="true" style="137" width="10.0"/>
+    <col min="6" max="6" customWidth="true" style="137" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="137" width="14.7109375"/>
+    <col min="8" max="8" customWidth="true" style="137" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="137" width="13.5703125"/>
+    <col min="10" max="11" customWidth="true" style="137" width="8.140625"/>
+    <col min="12" max="12" customWidth="true" style="137" width="8.0"/>
+    <col min="13" max="13" customWidth="true" style="137" width="13.85546875"/>
+    <col min="14" max="14" customWidth="true" style="137" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="137" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="137" width="14.7109375"/>
+    <col min="17" max="17" customWidth="true" style="137" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="137" width="9.0"/>
+    <col min="19" max="19" customWidth="true" style="137" width="10.85546875"/>
+    <col min="20" max="20" customWidth="true" style="137" width="17.85546875"/>
+    <col min="21" max="21" customWidth="true" style="137" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="137" width="11.5703125"/>
+    <col min="23" max="23" customWidth="true" style="137" width="9.28515625"/>
+    <col min="24" max="25" customWidth="true" style="137" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="137" width="11.28515625"/>
+    <col min="27" max="27" customWidth="true" style="137" width="12.0"/>
+    <col min="28" max="28" customWidth="true" style="137" width="12.28515625"/>
+    <col min="29" max="29" customWidth="true" style="137" width="14.7109375"/>
+    <col min="30" max="30" customWidth="true" style="163" width="12.28515625"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="163" width="13.5703125"/>
+    <col min="32" max="32" customWidth="true" style="163" width="13.5703125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="136" width="15.7109375"/>
+    <col min="34" max="34" customWidth="true" style="137" width="13.5703125"/>
+    <col min="35" max="35" customWidth="true" style="137" width="12.7109375"/>
+    <col min="36" max="16384" style="137" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -22868,43 +22868,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23338,43 +23338,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23926,43 +23926,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24396,43 +24396,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24866,43 +24866,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -25454,43 +25454,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -26042,43 +26042,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">

</xml_diff>

<commit_message>
Purchase Bill New Scenarios And DBSales Sheet Fixes
Purchase Bill New Scenarios And DBSales Sheet Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="47" activeTab="49"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="49" activeTab="51"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2693" uniqueCount="250">
   <si>
     <t>GST Sales</t>
   </si>
@@ -1822,43 +1822,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="14.0"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2410,43 +2410,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2984,44 +2984,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3447,44 +3447,44 @@
   <dimension ref="A1:AM13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="18.85546875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4075,44 +4075,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4538,44 +4538,44 @@
   <dimension ref="A1:AM36"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -6868,48 +6868,48 @@
   <dimension ref="A1:AQ6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="28" width="36.0"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="41" customWidth="true" style="29" width="14.140625"/>
-    <col min="42" max="42" customWidth="true" style="29" width="15.0"/>
-    <col min="43" max="43" customWidth="true" style="29" width="16.5703125"/>
-    <col min="44" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="36" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="41" width="14.140625" style="29" customWidth="1"/>
+    <col min="42" max="42" width="15" style="29" customWidth="1"/>
+    <col min="43" max="43" width="16.5703125" style="29" customWidth="1"/>
+    <col min="44" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
@@ -7365,43 +7365,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="34.5703125"/>
-    <col min="8" max="8" customWidth="true" style="29" width="21.28515625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.5703125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" style="29" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -7820,43 +7820,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8270,43 +8270,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8720,43 +8720,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9170,44 +9170,44 @@
   <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -9770,43 +9770,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10217,43 +10217,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10664,43 +10664,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -11123,42 +11123,42 @@
   <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="15.42578125"/>
-    <col min="38" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.42578125" style="29" customWidth="1"/>
+    <col min="38" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
@@ -11570,43 +11570,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12115,43 +12115,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
-    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
+    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12666,43 +12666,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
-    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
+    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13217,43 +13217,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
-    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
+    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13637,43 +13637,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
-    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
+    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14057,43 +14057,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="11.7109375"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
-    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="11.7109375" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
+    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14477,43 +14477,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -15065,44 +15065,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15528,44 +15528,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
-    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
-    <col min="40" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15991,12 +15991,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
-    <col min="6" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16061,12 +16061,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
-    <col min="6" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16131,17 +16131,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16286,17 +16286,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16441,15 +16441,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
-    <col min="7" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="14.85546875"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="29" customWidth="1"/>
+    <col min="7" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="14.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16594,15 +16594,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
-    <col min="7" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="29" customWidth="1"/>
+    <col min="7" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16747,17 +16747,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16902,17 +16902,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17057,43 +17057,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -17645,17 +17645,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17800,17 +17800,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17955,12 +17955,12 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18093,17 +18093,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18248,17 +18248,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
-    <col min="7" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
-    <col min="11" max="15" style="29" width="9.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
-    <col min="17" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
+    <col min="11" max="15" width="9.140625" style="29"/>
+    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18403,14 +18403,14 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="11.0"/>
-    <col min="11" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="11" style="29" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18543,45 +18543,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -18897,45 +18897,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19132,7 +19132,7 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" t="s" s="29">
+      <c r="C5" s="29" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -19141,13 +19141,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" t="s" s="29">
+      <c r="F5" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="G5" t="s" s="29">
+      <c r="G5" s="29" t="s">
         <v>167</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -19162,7 +19162,7 @@
         <f>I5*G5</f>
         <v>450</v>
       </c>
-      <c r="L5" t="s" s="29">
+      <c r="L5" s="29" t="s">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -19251,45 +19251,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19605,45 +19605,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19959,43 +19959,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -20547,45 +20547,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -20901,45 +20901,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -21136,7 +21136,7 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" t="s" s="29">
+      <c r="C5" s="29" t="s">
         <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -21145,13 +21145,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" t="s" s="29">
+      <c r="F5" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="G5" t="s" s="29">
+      <c r="G5" s="29" t="s">
         <v>220</v>
       </c>
-      <c r="H5" t="s" s="29">
+      <c r="H5" s="29" t="s">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -21166,7 +21166,7 @@
         <f>I5*G5</f>
         <v>400</v>
       </c>
-      <c r="L5" t="s" s="29">
+      <c r="L5" s="29" t="s">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -21255,18 +21255,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
-    <col min="11" max="14" style="29" width="9.140625"/>
-    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
-    <col min="16" max="16" style="29" width="9.140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
-    <col min="18" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="13" style="29" customWidth="1"/>
+    <col min="11" max="14" width="9.140625" style="29"/>
+    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="29"/>
+    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21350,7 +21350,7 @@
         <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="E5" s="67" t="s">
         <v>134</v>
@@ -21414,18 +21414,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
-    <col min="11" max="14" style="29" width="9.140625"/>
-    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
-    <col min="16" max="16" style="29" width="9.140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
-    <col min="18" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="13" style="29" customWidth="1"/>
+    <col min="11" max="14" width="9.140625" style="29"/>
+    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="29"/>
+    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21573,18 +21573,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
-    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
-    <col min="6" max="9" style="29" width="9.140625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
-    <col min="11" max="14" style="29" width="9.140625"/>
-    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
-    <col min="16" max="16" style="29" width="9.140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
-    <col min="18" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="29"/>
+    <col min="10" max="10" width="13" style="29" customWidth="1"/>
+    <col min="11" max="14" width="9.140625" style="29"/>
+    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="29"/>
+    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21732,9 +21732,9 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
-    <col min="3" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1">
@@ -21758,10 +21758,10 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" t="s" s="29">
+      <c r="A5" s="29" t="s">
         <v>234</v>
       </c>
-      <c r="B5" t="s" s="29">
+      <c r="B5" s="29" t="s">
         <v>232</v>
       </c>
     </row>
@@ -21783,13 +21783,13 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
-    <col min="3" max="3" customWidth="true" style="29" width="14.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="15.5703125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="7" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
@@ -21874,45 +21874,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
-    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
-    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
-    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
-    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
-    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
-    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
-    <col min="41" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
+    <col min="19" max="19" width="9" style="29" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
+    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
+    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
+    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
+    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -22228,40 +22228,40 @@
   <dimension ref="A1:AL8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="137" width="5.7109375"/>
-    <col min="2" max="2" customWidth="true" style="137" width="28.85546875"/>
-    <col min="3" max="3" customWidth="true" style="137" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="137" width="28.85546875"/>
-    <col min="5" max="5" customWidth="true" style="137" width="10.0"/>
-    <col min="6" max="6" customWidth="true" style="137" width="12.5703125"/>
-    <col min="7" max="7" customWidth="true" style="137" width="14.7109375"/>
-    <col min="8" max="8" customWidth="true" style="137" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="137" width="13.5703125"/>
-    <col min="10" max="11" customWidth="true" style="137" width="8.140625"/>
-    <col min="12" max="12" customWidth="true" style="137" width="8.0"/>
-    <col min="13" max="13" customWidth="true" style="137" width="13.85546875"/>
-    <col min="14" max="14" customWidth="true" style="137" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="137" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="137" width="14.7109375"/>
-    <col min="17" max="17" customWidth="true" style="137" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="137" width="9.0"/>
-    <col min="19" max="19" customWidth="true" style="137" width="10.85546875"/>
-    <col min="20" max="20" customWidth="true" style="137" width="17.85546875"/>
-    <col min="21" max="21" customWidth="true" style="137" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="137" width="11.5703125"/>
-    <col min="23" max="23" customWidth="true" style="137" width="9.28515625"/>
-    <col min="24" max="25" customWidth="true" style="137" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="137" width="11.28515625"/>
-    <col min="27" max="27" customWidth="true" style="137" width="12.0"/>
-    <col min="28" max="28" customWidth="true" style="137" width="12.28515625"/>
-    <col min="29" max="29" customWidth="true" style="137" width="14.7109375"/>
-    <col min="30" max="30" customWidth="true" style="163" width="12.28515625"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" style="163" width="13.5703125"/>
-    <col min="32" max="32" customWidth="true" style="163" width="13.5703125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" style="136" width="15.7109375"/>
-    <col min="34" max="34" customWidth="true" style="137" width="13.5703125"/>
-    <col min="35" max="35" customWidth="true" style="137" width="12.7109375"/>
-    <col min="36" max="16384" style="137" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="137" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="137" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="137" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="137" customWidth="1"/>
+    <col min="5" max="5" width="10" style="137" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="137" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="137" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="137" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="137" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="137" customWidth="1"/>
+    <col min="12" max="12" width="8" style="137" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="137" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="137" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="137" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="137" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="137" customWidth="1"/>
+    <col min="18" max="18" width="9" style="137" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="137" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="137" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="137" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" style="137" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="137" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="137" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="137" customWidth="1"/>
+    <col min="27" max="27" width="12" style="137" customWidth="1"/>
+    <col min="28" max="28" width="12.28515625" style="137" customWidth="1"/>
+    <col min="29" max="29" width="14.7109375" style="137" customWidth="1"/>
+    <col min="30" max="30" width="12.28515625" style="163" customWidth="1"/>
+    <col min="31" max="31" width="13.5703125" style="163" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.5703125" style="163" customWidth="1"/>
+    <col min="33" max="33" width="15.7109375" style="136" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.5703125" style="137" customWidth="1"/>
+    <col min="35" max="35" width="12.7109375" style="137" customWidth="1"/>
+    <col min="36" max="16384" width="9.140625" style="137"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -22868,43 +22868,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23338,43 +23338,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23926,43 +23926,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24396,43 +24396,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24866,43 +24866,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -25454,43 +25454,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -26042,43 +26042,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
-    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
-    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
-    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
-    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
-    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
-    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
-    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
-    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
-    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
-    <col min="35" max="35" style="29" width="9.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
-    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
-    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
-    <col min="39" max="16384" style="29" width="9.140625"/>
+    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
+    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" style="29" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
+    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
+    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
+    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" style="29"/>
+    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
+    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">

</xml_diff>

<commit_message>
Subcontract Closeshort Scenarios Added And Subcontract Order changes Fixes
Subcontract Closeshort Scenarios Added And Subcontract Order changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="49" activeTab="51"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="51" activeTab="51"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2693" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="250">
   <si>
     <t>GST Sales</t>
   </si>
@@ -1822,43 +1822,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="14.0"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2410,43 +2410,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -2984,44 +2984,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -3447,44 +3447,44 @@
   <dimension ref="A1:AM13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="18.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4075,44 +4075,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -4538,44 +4538,44 @@
   <dimension ref="A1:AM36"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -6868,48 +6868,48 @@
   <dimension ref="A1:AQ6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="36" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="41" width="14.140625" style="29" customWidth="1"/>
-    <col min="42" max="42" width="15" style="29" customWidth="1"/>
-    <col min="43" max="43" width="16.5703125" style="29" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="36.0"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="41" customWidth="true" style="29" width="14.140625"/>
+    <col min="42" max="42" customWidth="true" style="29" width="15.0"/>
+    <col min="43" max="43" customWidth="true" style="29" width="16.5703125"/>
+    <col min="44" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
@@ -7365,43 +7365,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.5703125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="21.28515625" style="29" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="34.5703125"/>
+    <col min="8" max="8" customWidth="true" style="29" width="21.28515625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -7820,43 +7820,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8270,43 +8270,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -8720,43 +8720,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -9170,44 +9170,44 @@
   <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -9770,43 +9770,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10217,43 +10217,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -10664,43 +10664,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -11123,42 +11123,42 @@
   <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.42578125" style="29" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="15.42578125"/>
+    <col min="38" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
@@ -11570,43 +11570,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12115,43 +12115,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -12666,43 +12666,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13217,43 +13217,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -13637,43 +13637,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14057,43 +14057,43 @@
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="11.7109375" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="54.5703125" style="29" customWidth="1"/>
-    <col min="38" max="38" width="34.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="11.7109375"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="54.5703125"/>
+    <col min="38" max="38" customWidth="true" style="29" width="34.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -14477,43 +14477,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -15065,44 +15065,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15528,44 +15528,44 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="12.5703125" style="28" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="29" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" customWidth="true" style="29" width="12.42578125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="28" width="12.5703125"/>
+    <col min="39" max="39" customWidth="true" style="29" width="15.42578125"/>
+    <col min="40" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -15991,12 +15991,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16061,12 +16061,12 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.42578125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
@@ -16131,17 +16131,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16286,17 +16286,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16441,15 +16441,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="14.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="14.85546875"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16594,15 +16594,15 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="29" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="12.0"/>
+    <col min="7" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16747,17 +16747,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -16902,17 +16902,17 @@
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="11.5703125"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17057,43 +17057,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -17645,17 +17645,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17800,17 +17800,17 @@
   <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="29" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.140625" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="20.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="13.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.140625"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="20.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -17955,12 +17955,12 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18093,17 +18093,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18248,17 +18248,17 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11.7109375" style="29" customWidth="1"/>
-    <col min="11" max="15" width="9.140625" style="29"/>
-    <col min="16" max="16" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="27.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="7" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.7109375"/>
+    <col min="11" max="15" style="29" width="9.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="12.140625"/>
+    <col min="17" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
@@ -18403,14 +18403,14 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="11" style="29" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="11.0"/>
+    <col min="11" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
@@ -18543,45 +18543,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -18897,45 +18897,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19251,45 +19251,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19605,45 +19605,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -19959,43 +19959,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -20547,45 +20547,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -20782,8 +20782,8 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>57</v>
+      <c r="C5" t="s" s="29">
+        <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -20791,13 +20791,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" t="s" s="29">
         <v>127</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>167</v>
-      </c>
-      <c r="H5" s="29" t="s">
+      <c r="G5" t="s" s="29">
+        <v>220</v>
+      </c>
+      <c r="H5" t="s" s="29">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -20812,7 +20812,7 @@
         <f>I5*G5</f>
         <v>450</v>
       </c>
-      <c r="L5" s="29" t="s">
+      <c r="L5" t="s" s="29">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -20901,45 +20901,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -21255,18 +21255,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21414,18 +21414,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21573,18 +21573,18 @@
   <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="29" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.140625" style="29"/>
-    <col min="10" max="10" width="13" style="29" customWidth="1"/>
-    <col min="11" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="10.42578125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="29"/>
-    <col min="17" max="17" width="20.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="21.7109375"/>
+    <col min="4" max="4" customWidth="true" style="29" width="24.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="19.5703125"/>
+    <col min="6" max="9" style="29" width="9.140625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="13.0"/>
+    <col min="11" max="14" style="29" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" style="29" width="10.42578125"/>
+    <col min="16" max="16" style="29" width="9.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="20.42578125"/>
+    <col min="18" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.75" customHeight="1">
@@ -21732,9 +21732,9 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
+    <col min="3" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1">
@@ -21758,10 +21758,10 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="29" t="s">
+      <c r="A5" t="s" s="29">
         <v>234</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" t="s" s="29">
         <v>232</v>
       </c>
     </row>
@@ -21783,13 +21783,13 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="15.28515625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.140625"/>
+    <col min="3" max="3" customWidth="true" style="29" width="14.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="15.5703125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="7" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
@@ -21874,45 +21874,45 @@
   <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="29" customWidth="1"/>
-    <col min="19" max="19" width="9" style="29" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.140625" style="29" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="29" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" style="29" customWidth="1"/>
-    <col min="30" max="30" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.28515625" style="29" customWidth="1"/>
-    <col min="33" max="33" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" style="36" customWidth="1"/>
-    <col min="35" max="35" width="10.28515625" style="28" customWidth="1"/>
-    <col min="36" max="36" width="12.42578125" style="29" customWidth="1"/>
-    <col min="37" max="37" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.140625" style="29" customWidth="1"/>
-    <col min="39" max="39" width="12.5703125" style="28" customWidth="1"/>
-    <col min="40" max="40" width="15.42578125" style="29" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" customWidth="true" style="29" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.28515625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="14.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="10" customWidth="true" style="29" width="13.5703125"/>
+    <col min="11" max="11" customWidth="true" style="29" width="12.28515625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.7109375"/>
+    <col min="19" max="19" customWidth="true" style="29" width="9.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="23" max="23" customWidth="true" style="29" width="16.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="25" max="26" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="27" max="27" customWidth="true" style="29" width="11.28515625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="29" max="29" customWidth="true" style="29" width="11.7109375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="32" max="32" customWidth="true" style="29" width="12.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="34" max="34" customWidth="true" style="36" width="14.140625"/>
+    <col min="35" max="35" customWidth="true" style="28" width="10.28515625"/>
+    <col min="36" max="36" customWidth="true" style="29" width="12.42578125"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="13.140625"/>
+    <col min="39" max="39" customWidth="true" style="28" width="12.5703125"/>
+    <col min="40" max="40" customWidth="true" style="29" width="15.42578125"/>
+    <col min="41" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
@@ -22228,40 +22228,40 @@
   <dimension ref="A1:AL8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="137" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="137" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="137" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="137" customWidth="1"/>
-    <col min="5" max="5" width="10" style="137" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="137" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="137" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="137" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="137" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="137" customWidth="1"/>
-    <col min="12" max="12" width="8" style="137" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="137" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="137" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="137" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="137" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="137" customWidth="1"/>
-    <col min="18" max="18" width="9" style="137" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="137" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="137" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="137" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" style="137" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="137" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="137" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="137" customWidth="1"/>
-    <col min="27" max="27" width="12" style="137" customWidth="1"/>
-    <col min="28" max="28" width="12.28515625" style="137" customWidth="1"/>
-    <col min="29" max="29" width="14.7109375" style="137" customWidth="1"/>
-    <col min="30" max="30" width="12.28515625" style="163" customWidth="1"/>
-    <col min="31" max="31" width="13.5703125" style="163" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.5703125" style="163" customWidth="1"/>
-    <col min="33" max="33" width="15.7109375" style="136" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.5703125" style="137" customWidth="1"/>
-    <col min="35" max="35" width="12.7109375" style="137" customWidth="1"/>
-    <col min="36" max="16384" width="9.140625" style="137"/>
+    <col min="1" max="1" customWidth="true" style="137" width="5.7109375"/>
+    <col min="2" max="2" customWidth="true" style="137" width="28.85546875"/>
+    <col min="3" max="3" customWidth="true" style="137" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="137" width="28.85546875"/>
+    <col min="5" max="5" customWidth="true" style="137" width="10.0"/>
+    <col min="6" max="6" customWidth="true" style="137" width="12.5703125"/>
+    <col min="7" max="7" customWidth="true" style="137" width="14.7109375"/>
+    <col min="8" max="8" customWidth="true" style="137" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="137" width="13.5703125"/>
+    <col min="10" max="11" customWidth="true" style="137" width="8.140625"/>
+    <col min="12" max="12" customWidth="true" style="137" width="8.0"/>
+    <col min="13" max="13" customWidth="true" style="137" width="13.85546875"/>
+    <col min="14" max="14" customWidth="true" style="137" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="137" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="137" width="14.7109375"/>
+    <col min="17" max="17" customWidth="true" style="137" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="137" width="9.0"/>
+    <col min="19" max="19" customWidth="true" style="137" width="10.85546875"/>
+    <col min="20" max="20" customWidth="true" style="137" width="17.85546875"/>
+    <col min="21" max="21" customWidth="true" style="137" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="137" width="11.5703125"/>
+    <col min="23" max="23" customWidth="true" style="137" width="9.28515625"/>
+    <col min="24" max="25" customWidth="true" style="137" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="137" width="11.28515625"/>
+    <col min="27" max="27" customWidth="true" style="137" width="12.0"/>
+    <col min="28" max="28" customWidth="true" style="137" width="12.28515625"/>
+    <col min="29" max="29" customWidth="true" style="137" width="14.7109375"/>
+    <col min="30" max="30" customWidth="true" style="163" width="12.28515625"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" style="163" width="13.5703125"/>
+    <col min="32" max="32" customWidth="true" style="163" width="13.5703125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" style="136" width="15.7109375"/>
+    <col min="34" max="34" customWidth="true" style="137" width="13.5703125"/>
+    <col min="35" max="35" customWidth="true" style="137" width="12.7109375"/>
+    <col min="36" max="16384" style="137" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -22868,43 +22868,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23338,43 +23338,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -23926,43 +23926,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24396,43 +24396,43 @@
   <dimension ref="A1:AL6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="28.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" style="28" width="11.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" style="29" width="26.85546875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -24866,43 +24866,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -25454,43 +25454,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
@@ -26042,43 +26042,43 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="29" customWidth="1"/>
-    <col min="10" max="11" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="29" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="29" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" style="29" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" style="29" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" style="29" customWidth="1"/>
-    <col min="29" max="29" width="16" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.28515625" style="29" customWidth="1"/>
-    <col min="32" max="32" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.140625" style="36" customWidth="1"/>
-    <col min="34" max="34" width="10.28515625" style="28" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="29"/>
-    <col min="36" max="36" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.28515625" style="29" customWidth="1"/>
-    <col min="38" max="38" width="15.42578125" style="29" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="5.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="29" width="30.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="29" width="4.5703125"/>
+    <col min="4" max="4" customWidth="true" style="29" width="29.85546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="29" width="10.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="29" width="12.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="10.140625"/>
+    <col min="9" max="9" customWidth="true" style="29" width="13.5703125"/>
+    <col min="10" max="11" bestFit="true" customWidth="true" style="29" width="8.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="29" width="8.0"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="29" width="13.85546875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="15" max="15" customWidth="true" style="29" width="12.5703125"/>
+    <col min="16" max="16" customWidth="true" style="29" width="14.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="29" width="9.7109375"/>
+    <col min="18" max="18" customWidth="true" style="29" width="9.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="10.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="17.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="29" width="10.5703125"/>
+    <col min="22" max="22" customWidth="true" style="29" width="16.140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="9.28515625"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="26" max="26" customWidth="true" style="29" width="11.28515625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" style="29" width="10.7109375"/>
+    <col min="28" max="28" customWidth="true" style="29" width="11.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" style="29" width="16.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="31" max="31" customWidth="true" style="29" width="12.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" style="29" width="14.7109375"/>
+    <col min="33" max="33" customWidth="true" style="36" width="14.140625"/>
+    <col min="34" max="34" customWidth="true" style="28" width="10.28515625"/>
+    <col min="35" max="35" style="29" width="9.140625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" style="29" width="13.140625"/>
+    <col min="37" max="37" customWidth="true" style="29" width="14.28515625"/>
+    <col min="38" max="38" customWidth="true" style="29" width="15.42578125"/>
+    <col min="39" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">

</xml_diff>

<commit_message>
Subcontract New Scenarios and Locators Fixes
Subcontract New Scenarios and Locators Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="51" activeTab="51"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="51" activeTab="55"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2780" uniqueCount="251">
   <si>
     <t>GST Sales</t>
   </si>
@@ -806,9 +806,6 @@
     <t>PROC- 5049</t>
   </si>
   <si>
-    <t>90856</t>
-  </si>
-  <si>
     <t>99830</t>
   </si>
   <si>
@@ -837,6 +834,12 @@
   </si>
   <si>
     <t>VR-SERIAL-FIFO-BATCH-80001QC</t>
+  </si>
+  <si>
+    <t>56071</t>
+  </si>
+  <si>
+    <t>SCO - Rework</t>
   </si>
 </sst>
 </file>
@@ -7277,7 +7280,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
@@ -7304,7 +7307,7 @@
         <v>175</v>
       </c>
       <c r="AO5" s="29" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -13071,7 +13074,7 @@
         <v>199</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -13199,7 +13202,7 @@
         <v>199</v>
       </c>
       <c r="AL6" s="66" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -15456,7 +15459,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -15919,7 +15922,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
@@ -16036,7 +16039,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>128</v>
@@ -19132,8 +19135,8 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>57</v>
+      <c r="C5" t="s" s="29">
+        <v>163</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -19141,13 +19144,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" t="s" s="29">
         <v>127</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>167</v>
-      </c>
-      <c r="H5" s="29" t="s">
+      <c r="G5" t="s" s="29">
+        <v>139</v>
+      </c>
+      <c r="H5" t="s" s="29">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -19162,7 +19165,7 @@
         <f>I5*G5</f>
         <v>450</v>
       </c>
-      <c r="L5" s="29" t="s">
+      <c r="L5" t="s" s="29">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -19499,7 +19502,7 @@
         <v>127</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H5" s="29" t="s">
         <v>160</v>
@@ -20782,7 +20785,7 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" t="s" s="29">
+      <c r="C5" s="29" t="s">
         <v>139</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -20791,13 +20794,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" t="s" s="29">
+      <c r="F5" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="G5" t="s" s="29">
-        <v>220</v>
-      </c>
-      <c r="H5" t="s" s="29">
+      <c r="G5" s="29" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" s="29" t="s">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -20812,7 +20815,7 @@
         <f>I5*G5</f>
         <v>450</v>
       </c>
-      <c r="L5" t="s" s="29">
+      <c r="L5" s="29" t="s">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -21136,8 +21139,8 @@
       <c r="B5" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>163</v>
+      <c r="C5" t="s" s="29">
+        <v>160</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -21145,13 +21148,13 @@
       <c r="E5" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="G5" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="H5" s="29" t="s">
+      <c r="F5" t="s" s="29">
+        <v>160</v>
+      </c>
+      <c r="G5" t="s" s="29">
+        <v>139</v>
+      </c>
+      <c r="H5" t="s" s="29">
         <v>160</v>
       </c>
       <c r="I5" s="10">
@@ -21166,7 +21169,7 @@
         <f>I5*G5</f>
         <v>400</v>
       </c>
-      <c r="L5" s="29" t="s">
+      <c r="L5" t="s" s="29">
         <v>32</v>
       </c>
       <c r="M5" s="33">
@@ -21344,7 +21347,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>139</v>
@@ -21503,7 +21506,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>139</v>
@@ -21759,7 +21762,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s" s="29">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B5" t="s" s="29">
         <v>232</v>
@@ -21814,6 +21817,10 @@
         <v>237</v>
       </c>
       <c r="F3" s="179"/>
+      <c r="G3" s="179" t="s">
+        <v>250</v>
+      </c>
+      <c r="H3" s="179"/>
     </row>
     <row r="4" spans="1:8" s="31" customFormat="1">
       <c r="A4" s="11" t="s">
@@ -21834,6 +21841,12 @@
       <c r="F4" s="11" t="s">
         <v>228</v>
       </c>
+      <c r="G4" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15">
       <c r="A5" s="122" t="s">
@@ -21854,15 +21867,22 @@
       <c r="F5" s="114" t="s">
         <v>160</v>
       </c>
+      <c r="G5" s="122" t="s">
+        <v>232</v>
+      </c>
+      <c r="H5" s="42" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="7" spans="1:8">
       <c r="H7" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23257,7 +23277,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -24315,7 +24335,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -24785,7 +24805,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>

</xml_diff>

<commit_message>
New Scenarios Of Cash Receipt And Bank Receipt Screen
New Scenarios Of Cash Receipt And Bank Receipt Screen And Updated The Locators Of RFQ
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2780" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2782" uniqueCount="253">
   <si>
     <t>GST Sales</t>
   </si>
@@ -840,6 +840,12 @@
   </si>
   <si>
     <t>SCO - Rework</t>
+  </si>
+  <si>
+    <t>54781</t>
+  </si>
+  <si>
+    <t>54766</t>
   </si>
 </sst>
 </file>
@@ -23276,8 +23282,8 @@
         <f t="shared" ref="AF5" si="1">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" s="36" t="s">
-        <v>245</v>
+      <c r="AG5" t="s" s="36">
+        <v>252</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>

</xml_diff>

<commit_message>
Finance Scenarios Added And Sales Invoices Fixes
Finance Scenarios Added And Sales Invoices Fixes
</commit_message>
<xml_diff>
--- a/testdata/DBSales.xlsx
+++ b/testdata/DBSales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="51" activeTab="55"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15525" windowHeight="6540" firstSheet="55" activeTab="61"/>
   </bookViews>
   <sheets>
     <sheet name="Domestic S&amp;D" sheetId="1" r:id="rId1"/>
@@ -68,6 +68,7 @@
     <sheet name="BRSPSI" sheetId="69" r:id="rId59"/>
     <sheet name="BRSPSIE" sheetId="70" r:id="rId60"/>
     <sheet name="BRSPMI" sheetId="71" r:id="rId61"/>
+    <sheet name="PurchaseBillDeviation" sheetId="74" r:id="rId62"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -87,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2782" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="265">
   <si>
     <t>GST Sales</t>
   </si>
@@ -704,9 +705,6 @@
     <t>81</t>
   </si>
   <si>
-    <t>99894</t>
-  </si>
-  <si>
     <t>Sales Order</t>
   </si>
   <si>
@@ -824,9 +822,6 @@
     <t>99175</t>
   </si>
   <si>
-    <t>91021</t>
-  </si>
-  <si>
     <t>93816</t>
   </si>
   <si>
@@ -842,10 +837,52 @@
     <t>SCO - Rework</t>
   </si>
   <si>
-    <t>54781</t>
+    <t>54766</t>
   </si>
   <si>
-    <t>54766</t>
+    <t>Scenario  :Purchase Bills deviation Calculation</t>
+  </si>
+  <si>
+    <t>Deviation</t>
+  </si>
+  <si>
+    <t>Matched Amt</t>
+  </si>
+  <si>
+    <t>GRN Amt</t>
+  </si>
+  <si>
+    <t>UnitCost</t>
+  </si>
+  <si>
+    <t>Proc.Qty</t>
+  </si>
+  <si>
+    <t>Curr.Matched Amt</t>
+  </si>
+  <si>
+    <t>Deviation Amt</t>
+  </si>
+  <si>
+    <t>375.00</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>99265</t>
+  </si>
+  <si>
+    <t>97795</t>
+  </si>
+  <si>
+    <t>97779</t>
+  </si>
+  <si>
+    <t>99260</t>
+  </si>
+  <si>
+    <t>45586</t>
   </si>
 </sst>
 </file>
@@ -1097,7 +1134,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="182">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1510,6 +1547,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1871,36 +1911,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -1947,10 +1987,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="2"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2220,7 +2260,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -2349,7 +2389,7 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -2459,36 +2499,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="52"/>
       <c r="AD1" s="52"/>
       <c r="AE1" s="52"/>
@@ -2535,10 +2575,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="51"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -2804,7 +2844,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>174</v>
+        <v>261</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -2928,7 +2968,7 @@
         <v>5</v>
       </c>
       <c r="AG6" s="36" t="s">
-        <v>174</v>
+        <v>260</v>
       </c>
       <c r="AH6" s="9">
         <f>AG6-AF6</f>
@@ -3034,36 +3074,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="80"/>
       <c r="AD1" s="80"/>
       <c r="AE1" s="80"/>
@@ -3110,10 +3150,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="79"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -3497,36 +3537,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="86"/>
       <c r="AD1" s="86"/>
       <c r="AE1" s="86"/>
@@ -3573,10 +3613,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="85"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4125,36 +4165,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="88"/>
       <c r="AD1" s="88"/>
       <c r="AE1" s="88"/>
@@ -4201,10 +4241,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="87"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -4588,36 +4628,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="93"/>
       <c r="AD1" s="93"/>
       <c r="AE1" s="93"/>
@@ -4664,10 +4704,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="92"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -6922,36 +6962,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -6998,10 +7038,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -7286,7 +7326,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="AH5" s="33">
         <f>AG5-AF5</f>
@@ -7313,7 +7353,7 @@
         <v>175</v>
       </c>
       <c r="AO5" s="29" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AP5" s="34">
         <f>AO5+AF5</f>
@@ -7414,36 +7454,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="133"/>
       <c r="AD1" s="133"/>
       <c r="AE1" s="133"/>
@@ -7490,10 +7530,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="132"/>
       <c r="D3" s="3">
         <v>4</v>
@@ -7869,36 +7909,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="54"/>
       <c r="AD1" s="54"/>
       <c r="AE1" s="54"/>
@@ -7945,10 +7985,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="53"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -8319,36 +8359,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -8395,10 +8435,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -8769,36 +8809,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -8845,10 +8885,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -9220,36 +9260,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="39"/>
       <c r="AD1" s="39"/>
       <c r="AE1" s="39"/>
@@ -9296,10 +9336,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="38"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -9819,36 +9859,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -9895,10 +9935,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -10266,36 +10306,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="56"/>
       <c r="AD1" s="56"/>
       <c r="AE1" s="56"/>
@@ -10342,10 +10382,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="55"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -10713,36 +10753,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -10789,10 +10829,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -11062,7 +11102,7 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -11171,36 +11211,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="62"/>
       <c r="AD1" s="62"/>
       <c r="AE1" s="62"/>
@@ -11247,10 +11287,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:37" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="61"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -11514,8 +11554,8 @@
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>15</v>
       </c>
-      <c r="AG5" s="36" t="s">
-        <v>190</v>
+      <c r="AG5" t="s" s="36">
+        <v>264</v>
       </c>
       <c r="AH5" s="9">
         <f>AG5-AF5</f>
@@ -11619,36 +11659,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="65"/>
       <c r="AD1" s="65"/>
       <c r="AE1" s="65"/>
@@ -11695,10 +11735,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="64"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -12164,36 +12204,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="69"/>
       <c r="AD1" s="69"/>
       <c r="AE1" s="69"/>
@@ -12240,10 +12280,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="68"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -12537,13 +12577,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C6" s="10">
         <v>0</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>32</v>
@@ -12715,36 +12755,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="71"/>
       <c r="AD1" s="71"/>
       <c r="AE1" s="71"/>
@@ -12791,10 +12831,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="70"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -12960,13 +13000,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>32</v>
@@ -13080,7 +13120,7 @@
         <v>199</v>
       </c>
       <c r="AL5" s="72" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:38" ht="15">
@@ -13208,7 +13248,7 @@
         <v>199</v>
       </c>
       <c r="AL6" s="66" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -13266,36 +13306,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="74"/>
       <c r="AD1" s="74"/>
       <c r="AE1" s="74"/>
@@ -13342,10 +13382,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="73"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -13686,36 +13726,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="76"/>
       <c r="AD1" s="76"/>
       <c r="AE1" s="76"/>
@@ -13762,10 +13802,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="75"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -14106,36 +14146,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="78"/>
       <c r="AD1" s="78"/>
       <c r="AE1" s="78"/>
@@ -14182,10 +14222,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="77"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -14526,36 +14566,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="41"/>
       <c r="AD1" s="41"/>
       <c r="AE1" s="41"/>
@@ -14602,10 +14642,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="40"/>
       <c r="D3" s="3">
         <v>2</v>
@@ -15115,36 +15155,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="84"/>
       <c r="AD1" s="84"/>
       <c r="AE1" s="84"/>
@@ -15191,10 +15231,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="83"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -15465,14 +15505,14 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>49586</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>173</v>
@@ -15578,36 +15618,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="82"/>
       <c r="AD1" s="82"/>
       <c r="AE1" s="82"/>
@@ -15654,10 +15694,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:39" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="81"/>
       <c r="D3" s="3">
         <v>1</v>
@@ -15928,14 +15968,14 @@
         <v>15</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AH5" s="34">
         <f>AG5-AF5</f>
         <v>65983</v>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>173</v>
@@ -16009,19 +16049,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -16045,7 +16085,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>128</v>
@@ -16079,19 +16119,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:5" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:5" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -16115,7 +16155,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>127</v>
@@ -16154,19 +16194,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="165"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="164"/>
       <c r="D3" s="164"/>
     </row>
@@ -16271,7 +16311,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16309,19 +16349,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -16426,7 +16466,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16462,19 +16502,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="168"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="167"/>
       <c r="D3" s="167"/>
     </row>
@@ -16579,7 +16619,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -16615,19 +16655,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -16770,19 +16810,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="165"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="164"/>
       <c r="D3" s="164"/>
     </row>
@@ -16887,7 +16927,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="166" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -16925,19 +16965,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="119"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="118"/>
       <c r="D3" s="118"/>
     </row>
@@ -17042,7 +17082,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -17106,36 +17146,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
-      <c r="R1" s="177"/>
-      <c r="S1" s="177"/>
-      <c r="T1" s="177"/>
-      <c r="U1" s="177"/>
-      <c r="V1" s="177"/>
-      <c r="W1" s="177"/>
-      <c r="X1" s="177"/>
-      <c r="Y1" s="177"/>
-      <c r="Z1" s="177"/>
-      <c r="AA1" s="177"/>
-      <c r="AB1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
+      <c r="Q1" s="178"/>
+      <c r="R1" s="178"/>
+      <c r="S1" s="178"/>
+      <c r="T1" s="178"/>
+      <c r="U1" s="178"/>
+      <c r="V1" s="178"/>
+      <c r="W1" s="178"/>
+      <c r="X1" s="178"/>
+      <c r="Y1" s="178"/>
+      <c r="Z1" s="178"/>
+      <c r="AA1" s="178"/>
+      <c r="AB1" s="178"/>
       <c r="AC1" s="44"/>
       <c r="AD1" s="44"/>
       <c r="AE1" s="44"/>
@@ -17182,10 +17222,10 @@
       <c r="AG2" s="27"/>
     </row>
     <row r="3" spans="1:38" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="177"/>
       <c r="C3" s="43"/>
       <c r="D3" s="3">
         <v>3</v>
@@ -17668,19 +17708,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="165"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="164"/>
       <c r="D3" s="164"/>
     </row>
@@ -17785,7 +17825,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17823,19 +17863,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -17940,7 +17980,7 @@
         <v>88363221</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -17973,19 +18013,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:15" ht="18">
       <c r="D2" s="112"/>
     </row>
     <row r="3" spans="1:15" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="111"/>
       <c r="D3" s="111"/>
     </row>
@@ -18116,19 +18156,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="168"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="167"/>
       <c r="D3" s="167"/>
     </row>
@@ -18271,19 +18311,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:16" ht="18">
       <c r="D2" s="121"/>
     </row>
     <row r="3" spans="1:16" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="120"/>
       <c r="D3" s="120"/>
     </row>
@@ -18423,19 +18463,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
     </row>
     <row r="2" spans="1:15" ht="18">
       <c r="D2" s="117"/>
     </row>
     <row r="3" spans="1:15" ht="19.899999999999999" customHeight="1">
-      <c r="A3" s="176"/>
-      <c r="B3" s="176"/>
+      <c r="A3" s="177"/>
+      <c r="B3" s="177"/>
       <c r="C3" s="116"/>
       <c r="D3" s="116"/>
     </row>
@@ -18594,37 +18634,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="27.75" customHeight="1">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="178" t="s">
         <v>166</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"